<commit_message>
Add DataCamp evidence to portfolio
</commit_message>
<xml_diff>
--- a/public/Integraal_Sprint_Logboek_Officieel.xlsx
+++ b/public/Integraal_Sprint_Logboek_Officieel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasmijnmesu/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4D3B963-0ABD-2B4E-B6FD-D55C4244B890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5AE274C6-02B1-D24C-9FDD-BC962E88A980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10500" yWindow="760" windowWidth="18900" windowHeight="17360" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10500" yWindow="760" windowWidth="18900" windowHeight="17320" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -277,11 +277,6 @@
 zodat ik kan onderbouwen of en hoe een agentic aanpak waarde toevoegt aan mijn specifieke minoroplossing.</t>
   </si>
   <si>
-    <t>1. DataCamp-cursus "Introduction to AI Agents" succesvol afgerond, inclusief certificaat/bewijs van afronding in logboek.
-2. Een geschreven analyse (ca. 300–500 woorden) met vergelijking tussen de huidige aanpak en een agentic aanpak voor de eigen opdracht.
-3. Minimaal 2 relevante verdiepingsvideo's bekeken en gedocumenteerd met titel, link en korte kernboodschap.</t>
-  </si>
-  <si>
     <t>1. Betrouwbaarheid &amp; herkomst: gebruik van actuele, gereputeerde bronnen en correcte bronvermelding.
 2. Diepgang &amp; onderbouwing: helder onderscheid gemaakt tussen eenvoudige prompt-chains/workflows en daadwerkelijke autonome agents.
 3. Toepasbaarheid: de vertaalslag sluit direct aan op de context van het eigen projectportfolio.</t>
@@ -290,11 +285,6 @@
     <t>Als AI-projectmanager in opleiding,
 wil ik de bedrijfsactiviteiten, laadinfrastructuur-diensten en potentiële AI-kansen van Blue Current onderzoeken,
 zodat ik tijdens het eerste intakegesprek direct gerichte AI-use cases kan pitchen en een scherpe minoropdracht kan formuleren (Leeruitkomst: Impact &amp; Oplossing).</t>
-  </si>
-  <si>
-    <t>1. Een compact onderzoeksverslag (1 à 2 pagina's in logboek/Notion) met daarin de kernactiviteiten en propositie van Blue Current, en de huidige technologie- en laadinfrastructuurcontext.
-2. Minimaal 3 concrete AI-kansen/use cases uitgewerkt (bijv. slim laden/netcongestie, voorspellend onderhoud, geautomatiseerde support).
-3. Een gestructureerde vragenlijst (5–8 vragen) voor het intakegesprek met Blue Current.</t>
   </si>
   <si>
     <t>1. Bronnen &amp; herkomst: relevante openbare bronnen gebruikt (website, nieuws, LinkedIn) met expliciete bronvermelding.
@@ -373,6 +363,16 @@
   </si>
   <si>
     <t>O</t>
+  </si>
+  <si>
+    <t>1. Een compact onderzoeksverslag met daarin de kernactiviteiten en propositie van Blue Current, en de huidige technologie- en laadinfrastructuurcontext.
+2. Minimaal 3 concrete AI-kansen/use cases uitgewerkt (bijv. slim laden/netcongestie, voorspellend onderhoud, geautomatiseerde support).
+3. Een gestructureerde vragenlijst (5–8 vragen) voor het intakegesprek met Blue Current.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. DataCamp-cursus "Introduction to AI Agents" succesvol afgerond, inclusief certificaat/bewijs van afronding in logboek.
+2. Een geschreven samenvatting waar de stof besproken wordt en je ten alle tijden de stof terug kan vinden
+3. De samenvatting is toegevoegd aan mijn portfolio om deze altijd bij de hand te hebben. </t>
   </si>
 </sst>
 </file>
@@ -984,12 +984,6 @@
   </cellStyleXfs>
   <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1239,6 +1233,12 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1944,325 +1944,325 @@
     <col min="1" max="1" width="14.5" customWidth="1"/>
     <col min="2" max="2" width="6.5" customWidth="1"/>
     <col min="3" max="3" width="9.5" customWidth="1"/>
-    <col min="4" max="11" width="9.1640625" style="5" customWidth="1"/>
+    <col min="4" max="11" width="9.1640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="8">
         <v>2</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="8">
         <f>COUNTIF(D2:K2, "V")</f>
         <v>1</v>
       </c>
-      <c r="D2" s="13" t="str">
+      <c r="D2" s="9" t="str">
         <f>Logboek!C18</f>
         <v>V</v>
       </c>
-      <c r="E2" s="13" t="str">
+      <c r="E2" s="9" t="str">
         <f>Logboek!C46</f>
         <v>-</v>
       </c>
-      <c r="F2" s="13" t="str">
+      <c r="F2" s="9" t="str">
         <f>Logboek!C74</f>
         <v>-</v>
       </c>
-      <c r="G2" s="13" t="str">
+      <c r="G2" s="9" t="str">
         <f>Logboek!C102</f>
         <v>-</v>
       </c>
-      <c r="H2" s="13" t="str">
+      <c r="H2" s="9" t="str">
         <f>Logboek!C130</f>
         <v>-</v>
       </c>
-      <c r="I2" s="13" t="str">
+      <c r="I2" s="9" t="str">
         <f>Logboek!C158</f>
         <v>-</v>
       </c>
-      <c r="J2" s="13" t="str">
+      <c r="J2" s="9" t="str">
         <f>Logboek!C186</f>
         <v>-</v>
       </c>
-      <c r="K2" s="14" t="str">
+      <c r="K2" s="10" t="str">
         <f>Logboek!C214</f>
         <v>-</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="8">
         <v>4</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="8">
         <f>COUNTIF(D3:K3, "V")</f>
         <v>2</v>
       </c>
-      <c r="D3" s="13" t="str">
+      <c r="D3" s="9" t="str">
         <f>Logboek!C19</f>
         <v>V</v>
       </c>
-      <c r="E3" s="13" t="str">
+      <c r="E3" s="9" t="str">
         <f>Logboek!C47</f>
         <v>V</v>
       </c>
-      <c r="F3" s="13" t="str">
+      <c r="F3" s="9" t="str">
         <f>Logboek!C75</f>
         <v>-</v>
       </c>
-      <c r="G3" s="13" t="str">
+      <c r="G3" s="9" t="str">
         <f>Logboek!C103</f>
         <v>-</v>
       </c>
-      <c r="H3" s="13" t="str">
+      <c r="H3" s="9" t="str">
         <f>Logboek!C131</f>
         <v>-</v>
       </c>
-      <c r="I3" s="13" t="str">
+      <c r="I3" s="9" t="str">
         <f>Logboek!C159</f>
         <v>-</v>
       </c>
-      <c r="J3" s="13" t="str">
+      <c r="J3" s="9" t="str">
         <f>Logboek!C187</f>
         <v>-</v>
       </c>
-      <c r="K3" s="14" t="str">
+      <c r="K3" s="10" t="str">
         <f>Logboek!C215</f>
         <v>-</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="8">
         <v>2</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="8">
         <f>COUNTIF(D4:K4, "V")</f>
         <v>0</v>
       </c>
-      <c r="D4" s="13" t="str">
+      <c r="D4" s="9" t="str">
         <f>Logboek!C20</f>
         <v>-</v>
       </c>
-      <c r="E4" s="13" t="str">
+      <c r="E4" s="9" t="str">
         <f>Logboek!C48</f>
         <v>-</v>
       </c>
-      <c r="F4" s="13" t="str">
+      <c r="F4" s="9" t="str">
         <f>Logboek!C76</f>
         <v>-</v>
       </c>
-      <c r="G4" s="13" t="str">
+      <c r="G4" s="9" t="str">
         <f>Logboek!C104</f>
         <v>-</v>
       </c>
-      <c r="H4" s="13" t="str">
+      <c r="H4" s="9" t="str">
         <f>Logboek!C132</f>
         <v>-</v>
       </c>
-      <c r="I4" s="13" t="str">
+      <c r="I4" s="9" t="str">
         <f>Logboek!C160</f>
         <v>-</v>
       </c>
-      <c r="J4" s="13" t="str">
+      <c r="J4" s="9" t="str">
         <f>Logboek!C188</f>
         <v>-</v>
       </c>
-      <c r="K4" s="14" t="str">
+      <c r="K4" s="10" t="str">
         <f>Logboek!C216</f>
         <v>-</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="8">
         <v>4</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="8">
         <f>COUNTIF(D5:K5, "V")</f>
         <v>2</v>
       </c>
-      <c r="D5" s="13" t="str">
+      <c r="D5" s="9" t="str">
         <f>Logboek!C21</f>
         <v>V</v>
       </c>
-      <c r="E5" s="13" t="str">
+      <c r="E5" s="9" t="str">
         <f>Logboek!C49</f>
         <v>V</v>
       </c>
-      <c r="F5" s="13" t="str">
+      <c r="F5" s="9" t="str">
         <f>Logboek!C77</f>
         <v>-</v>
       </c>
-      <c r="G5" s="13" t="str">
+      <c r="G5" s="9" t="str">
         <f>Logboek!C105</f>
         <v>-</v>
       </c>
-      <c r="H5" s="13" t="str">
+      <c r="H5" s="9" t="str">
         <f>Logboek!C133</f>
         <v>-</v>
       </c>
-      <c r="I5" s="13" t="str">
+      <c r="I5" s="9" t="str">
         <f>Logboek!C161</f>
         <v>-</v>
       </c>
-      <c r="J5" s="13" t="str">
+      <c r="J5" s="9" t="str">
         <f>Logboek!C189</f>
         <v>-</v>
       </c>
-      <c r="K5" s="14" t="str">
+      <c r="K5" s="10" t="str">
         <f>Logboek!C217</f>
         <v>-</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="8">
         <v>6</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="8">
         <f>COUNTIF(D6:K6, "V")</f>
         <v>2</v>
       </c>
-      <c r="D6" s="13" t="str">
+      <c r="D6" s="9" t="str">
         <f>Logboek!C22</f>
         <v>V</v>
       </c>
-      <c r="E6" s="13" t="str">
+      <c r="E6" s="9" t="str">
         <f>Logboek!C50</f>
         <v>V</v>
       </c>
-      <c r="F6" s="13" t="str">
+      <c r="F6" s="9" t="str">
         <f>Logboek!C78</f>
         <v>-</v>
       </c>
-      <c r="G6" s="13" t="str">
+      <c r="G6" s="9" t="str">
         <f>Logboek!C106</f>
         <v>-</v>
       </c>
-      <c r="H6" s="13" t="str">
+      <c r="H6" s="9" t="str">
         <f>Logboek!C134</f>
         <v>-</v>
       </c>
-      <c r="I6" s="13" t="str">
+      <c r="I6" s="9" t="str">
         <f>Logboek!C162</f>
         <v>-</v>
       </c>
-      <c r="J6" s="13" t="str">
+      <c r="J6" s="9" t="str">
         <f>Logboek!C190</f>
         <v>-</v>
       </c>
-      <c r="K6" s="14" t="str">
+      <c r="K6" s="10" t="str">
         <f>Logboek!C218</f>
         <v>-</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="12">
         <f>SUM(B2:B6)</f>
         <v>18</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="12">
         <f>SUM(D6:K7)</f>
         <v>7</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="13">
         <f t="shared" ref="D7:K7" si="0">COUNTIF(D2:D6, "V")</f>
         <v>4</v>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="13">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="13">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="13">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="13">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I7" s="17">
+      <c r="I7" s="13">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J7" s="17">
+      <c r="J7" s="13">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K7" s="18">
+      <c r="K7" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="106" t="s">
+      <c r="B9" s="102" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
+      <c r="C9" s="103"/>
+      <c r="D9" s="103"/>
+      <c r="E9" s="103"/>
+      <c r="F9" s="103"/>
+      <c r="G9" s="103"/>
+      <c r="H9" s="103"/>
+      <c r="I9" s="103"/>
+      <c r="J9" s="103"/>
+      <c r="K9" s="103"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2296,2206 +2296,2206 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="106" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="20"/>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
+      <c r="A2" s="16"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22" t="s">
+      <c r="B3" s="17"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="21" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="168" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="24" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="162.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="24" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="156.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="24" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="26"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="28"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="24"/>
     </row>
     <row r="9" spans="1:4" ht="43.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="30"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="32"/>
-      <c r="D9" s="33"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="29"/>
     </row>
     <row r="10" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="21" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="35"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="38"/>
+      <c r="A13" s="31"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="34"/>
     </row>
     <row r="14" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="39"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="38"/>
+      <c r="A14" s="35"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="34"/>
     </row>
     <row r="15" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="41"/>
-      <c r="B15" s="41"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
     </row>
     <row r="16" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="25" t="s">
+      <c r="D17" s="21" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="148.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="37" t="s">
+      <c r="B18" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="44" t="s">
+      <c r="C18" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="24" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="36.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="43" t="s">
+      <c r="A19" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="37" t="s">
+      <c r="B19" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="44" t="s">
+      <c r="C19" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="28" t="s">
+      <c r="D19" s="24" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="43" t="s">
+      <c r="A20" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="44" t="s">
+      <c r="C20" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="24" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="192.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="37" t="s">
+      <c r="B21" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="44" t="s">
+      <c r="C21" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="28" t="s">
+      <c r="D21" s="24" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="207.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="45" t="s">
+      <c r="A22" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="46" t="s">
+      <c r="B22" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="47" t="s">
+      <c r="C22" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="29" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="20"/>
-      <c r="B23" s="48"/>
-      <c r="C23" s="49"/>
-      <c r="D23" s="49"/>
+      <c r="A23" s="16"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="45"/>
+      <c r="D23" s="45"/>
     </row>
     <row r="24" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B24" s="50"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="47"/>
     </row>
     <row r="25" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B25" s="52" t="s">
+      <c r="B25" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="53" t="s">
+      <c r="C25" s="49" t="s">
         <v>65</v>
       </c>
-      <c r="D25" s="25" t="s">
+      <c r="D25" s="21" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="35"/>
-      <c r="B26" s="27"/>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
+      <c r="A26" s="31"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="50"/>
+      <c r="D26" s="50"/>
     </row>
     <row r="27" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="55"/>
-      <c r="B27" s="56"/>
-      <c r="C27" s="54"/>
-      <c r="D27" s="54"/>
+      <c r="A27" s="51"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="50"/>
     </row>
     <row r="28" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="41"/>
-      <c r="B28" s="41"/>
-      <c r="C28" s="41"/>
-      <c r="D28" s="41"/>
+      <c r="A28" s="37"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
     </row>
     <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="104" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
+      <c r="B29" s="104"/>
+      <c r="C29" s="104"/>
+      <c r="D29" s="104"/>
     </row>
     <row r="30" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="57"/>
-      <c r="B30" s="57"/>
-      <c r="C30" s="57"/>
-      <c r="D30" s="57"/>
+      <c r="A30" s="53"/>
+      <c r="B30" s="53"/>
+      <c r="C30" s="53"/>
+      <c r="D30" s="53"/>
     </row>
     <row r="31" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="58" t="s">
+      <c r="A31" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="B31" s="58"/>
-      <c r="C31" s="58"/>
-      <c r="D31" s="22" t="s">
+      <c r="B31" s="54"/>
+      <c r="C31" s="54"/>
+      <c r="D31" s="18" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="59" t="s">
+      <c r="A32" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="B32" s="60" t="s">
+      <c r="B32" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="C32" s="60" t="s">
+      <c r="C32" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="D32" s="61" t="s">
+      <c r="D32" s="57" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="141" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="62" t="s">
+      <c r="A33" s="58" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="63" t="s">
+      <c r="B33" s="59" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="64" t="s">
+      <c r="C33" s="60" t="s">
+        <v>95</v>
+      </c>
+      <c r="D33" s="61" t="s">
         <v>70</v>
       </c>
-      <c r="D33" s="65" t="s">
+    </row>
+    <row r="34" spans="1:4" ht="143" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="58" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34" s="59" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" ht="143" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="62" t="s">
-        <v>26</v>
-      </c>
-      <c r="B34" s="63" t="s">
+      <c r="C34" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="D34" s="61" t="s">
         <v>72</v>
       </c>
-      <c r="C34" s="64" t="s">
+    </row>
+    <row r="35" spans="1:4" ht="125" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="58" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="D34" s="65" t="s">
+      <c r="C35" s="60" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" ht="125" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="62" t="s">
+      <c r="D35" s="61" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="58"/>
+      <c r="B36" s="59"/>
+      <c r="C36" s="60"/>
+      <c r="D36" s="61"/>
+    </row>
+    <row r="37" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="62"/>
+      <c r="B37" s="63"/>
+      <c r="C37" s="64"/>
+      <c r="D37" s="65"/>
+    </row>
+    <row r="38" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="53"/>
+      <c r="B38" s="53"/>
+      <c r="C38" s="53"/>
+      <c r="D38" s="53"/>
+    </row>
+    <row r="39" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="54" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" s="54"/>
+      <c r="C39" s="54"/>
+      <c r="D39" s="54"/>
+    </row>
+    <row r="40" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="56" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="D40" s="57" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="66">
+        <v>46288</v>
+      </c>
+      <c r="B41" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="C41" s="60" t="s">
+        <v>79</v>
+      </c>
+      <c r="D41" s="61" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="82.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="67">
+        <v>46292</v>
+      </c>
+      <c r="B42" s="68" t="s">
+        <v>81</v>
+      </c>
+      <c r="C42" s="68" t="s">
+        <v>82</v>
+      </c>
+      <c r="D42" s="69" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="70"/>
+      <c r="B43" s="71"/>
+      <c r="C43" s="71"/>
+      <c r="D43" s="72"/>
+    </row>
+    <row r="44" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="73" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" s="73"/>
+      <c r="C44" s="73"/>
+      <c r="D44" s="73"/>
+    </row>
+    <row r="45" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="B45" s="56" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" s="56" t="s">
+        <v>45</v>
+      </c>
+      <c r="D45" s="57" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="74" t="s">
+        <v>47</v>
+      </c>
+      <c r="B46" s="75" t="s">
+        <v>48</v>
+      </c>
+      <c r="C46" s="76" t="s">
+        <v>56</v>
+      </c>
+      <c r="D46" s="61"/>
+    </row>
+    <row r="47" spans="1:4" ht="170" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="74" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="75" t="s">
+        <v>52</v>
+      </c>
+      <c r="C47" s="76" t="s">
+        <v>49</v>
+      </c>
+      <c r="D47" s="61" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="74" t="s">
+        <v>54</v>
+      </c>
+      <c r="B48" s="75" t="s">
+        <v>55</v>
+      </c>
+      <c r="C48" s="76" t="s">
+        <v>56</v>
+      </c>
+      <c r="D48" s="61"/>
+    </row>
+    <row r="49" spans="1:4" ht="169" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="74" t="s">
+        <v>57</v>
+      </c>
+      <c r="B49" s="75" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" s="76" t="s">
+        <v>49</v>
+      </c>
+      <c r="D49" s="61" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="175" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="77" t="s">
+        <v>60</v>
+      </c>
+      <c r="B50" s="78" t="s">
+        <v>61</v>
+      </c>
+      <c r="C50" s="79" t="s">
+        <v>49</v>
+      </c>
+      <c r="D50" s="65" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="53"/>
+      <c r="B51" s="80"/>
+      <c r="C51" s="81"/>
+      <c r="D51" s="81"/>
+    </row>
+    <row r="52" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="54" t="s">
+        <v>63</v>
+      </c>
+      <c r="B52" s="82"/>
+      <c r="C52" s="83"/>
+      <c r="D52" s="83"/>
+    </row>
+    <row r="53" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="B53" s="84" t="s">
+        <v>64</v>
+      </c>
+      <c r="C53" s="85" t="s">
+        <v>65</v>
+      </c>
+      <c r="D53" s="57" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="66"/>
+      <c r="B54" s="60"/>
+      <c r="C54" s="60"/>
+      <c r="D54" s="61"/>
+    </row>
+    <row r="55" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="86"/>
+      <c r="B55" s="87"/>
+      <c r="C55" s="68"/>
+      <c r="D55" s="69"/>
+    </row>
+    <row r="56" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="70"/>
+      <c r="B56" s="71"/>
+      <c r="C56" s="71"/>
+      <c r="D56" s="72"/>
+    </row>
+    <row r="57" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="105" t="s">
+        <v>87</v>
+      </c>
+      <c r="B57" s="105"/>
+      <c r="C57" s="105"/>
+      <c r="D57" s="105"/>
+    </row>
+    <row r="58" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="16"/>
+      <c r="B58" s="16"/>
+      <c r="C58" s="16"/>
+      <c r="D58" s="16"/>
+    </row>
+    <row r="59" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B59" s="17"/>
+      <c r="C59" s="17"/>
+      <c r="D59" s="18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B60" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="C60" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60" s="21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="63" t="s">
-        <v>75</v>
-      </c>
-      <c r="C35" s="64" t="s">
+      <c r="B61" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="D35" s="65" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="62"/>
-      <c r="B36" s="63"/>
-      <c r="C36" s="64"/>
-      <c r="D36" s="65"/>
-    </row>
-    <row r="37" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="66"/>
-      <c r="B37" s="67"/>
-      <c r="C37" s="68"/>
-      <c r="D37" s="69"/>
-    </row>
-    <row r="38" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="57"/>
-      <c r="B38" s="57"/>
-      <c r="C38" s="57"/>
-      <c r="D38" s="57"/>
-    </row>
-    <row r="39" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="58" t="s">
+      <c r="C61" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D61" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="22"/>
+      <c r="B62" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C62" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D62" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="22"/>
+      <c r="B63" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C63" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D63" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="22"/>
+      <c r="B64" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C64" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D64" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="26"/>
+      <c r="B65" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="C65" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D65" s="29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="16"/>
+      <c r="B66" s="16"/>
+      <c r="C66" s="16"/>
+      <c r="D66" s="16"/>
+    </row>
+    <row r="67" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="58"/>
-      <c r="C39" s="58"/>
-      <c r="D39" s="58"/>
-    </row>
-    <row r="40" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="59" t="s">
+      <c r="B67" s="17"/>
+      <c r="C67" s="17"/>
+      <c r="D67" s="17"/>
+    </row>
+    <row r="68" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="60" t="s">
+      <c r="B68" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C40" s="60" t="s">
+      <c r="C68" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="D40" s="61" t="s">
+      <c r="D68" s="21" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="70">
-        <v>46288</v>
-      </c>
-      <c r="B41" s="64" t="s">
-        <v>80</v>
-      </c>
-      <c r="C41" s="64" t="s">
-        <v>81</v>
-      </c>
-      <c r="D41" s="65" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="82.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="71">
-        <v>46292</v>
-      </c>
-      <c r="B42" s="72" t="s">
-        <v>83</v>
-      </c>
-      <c r="C42" s="72" t="s">
-        <v>84</v>
-      </c>
-      <c r="D42" s="73" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="74"/>
-      <c r="B43" s="75"/>
-      <c r="C43" s="75"/>
-      <c r="D43" s="76"/>
-    </row>
-    <row r="44" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="77" t="s">
+    <row r="69" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="31"/>
+      <c r="B69" s="23"/>
+      <c r="C69" s="23"/>
+      <c r="D69" s="24"/>
+    </row>
+    <row r="70" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="35"/>
+      <c r="B70" s="88"/>
+      <c r="C70" s="88"/>
+      <c r="D70" s="89"/>
+    </row>
+    <row r="71" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="90"/>
+      <c r="B71" s="37"/>
+      <c r="C71" s="37"/>
+      <c r="D71" s="91"/>
+    </row>
+    <row r="72" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="77"/>
-      <c r="C44" s="77"/>
-      <c r="D44" s="77"/>
-    </row>
-    <row r="45" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="59" t="s">
+      <c r="B72" s="38"/>
+      <c r="C72" s="38"/>
+      <c r="D72" s="38"/>
+    </row>
+    <row r="73" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B45" s="60" t="s">
+      <c r="B73" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C45" s="60" t="s">
+      <c r="C73" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D45" s="61" t="s">
+      <c r="D73" s="21" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="78" t="s">
+    <row r="74" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="B46" s="79" t="s">
+      <c r="B74" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="C46" s="80" t="s">
+      <c r="C74" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D46" s="65"/>
-    </row>
-    <row r="47" spans="1:4" ht="170" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="78" t="s">
+      <c r="D74" s="24"/>
+    </row>
+    <row r="75" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B47" s="79" t="s">
+      <c r="B75" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="C47" s="80" t="s">
-        <v>49</v>
-      </c>
-      <c r="D47" s="65" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="78" t="s">
+      <c r="C75" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="D75" s="24"/>
+    </row>
+    <row r="76" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="B48" s="79" t="s">
+      <c r="B76" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="C48" s="80" t="s">
+      <c r="C76" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D48" s="65"/>
-    </row>
-    <row r="49" spans="1:4" ht="169" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="78" t="s">
+      <c r="D76" s="24"/>
+    </row>
+    <row r="77" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="B49" s="79" t="s">
+      <c r="B77" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="C49" s="80" t="s">
-        <v>49</v>
-      </c>
-      <c r="D49" s="65" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="175" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="81" t="s">
+      <c r="C77" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="D77" s="24"/>
+    </row>
+    <row r="78" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="B50" s="82" t="s">
+      <c r="B78" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="C50" s="83" t="s">
-        <v>49</v>
-      </c>
-      <c r="D50" s="69" t="s">
+      <c r="C78" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="D78" s="29"/>
+    </row>
+    <row r="79" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="16"/>
+      <c r="B79" s="44"/>
+      <c r="C79" s="45"/>
+      <c r="D79" s="45"/>
+    </row>
+    <row r="80" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B80" s="46"/>
+      <c r="C80" s="47"/>
+      <c r="D80" s="47"/>
+    </row>
+    <row r="81" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B81" s="48" t="s">
+        <v>64</v>
+      </c>
+      <c r="C81" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="D81" s="21" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="31"/>
+      <c r="B82" s="23"/>
+      <c r="C82" s="50"/>
+      <c r="D82" s="50"/>
+    </row>
+    <row r="83" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="51"/>
+      <c r="B83" s="92"/>
+      <c r="C83" s="50"/>
+      <c r="D83" s="50"/>
+    </row>
+    <row r="84" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="90"/>
+      <c r="B84" s="37"/>
+      <c r="C84" s="37"/>
+      <c r="D84" s="91"/>
+    </row>
+    <row r="85" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="104" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="57"/>
-      <c r="B51" s="84"/>
-      <c r="C51" s="85"/>
-      <c r="D51" s="85"/>
-    </row>
-    <row r="52" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="58" t="s">
+      <c r="B85" s="104"/>
+      <c r="C85" s="104"/>
+      <c r="D85" s="104"/>
+    </row>
+    <row r="86" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="53"/>
+      <c r="B86" s="53"/>
+      <c r="C86" s="53"/>
+      <c r="D86" s="53"/>
+    </row>
+    <row r="87" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="B87" s="54"/>
+      <c r="C87" s="54"/>
+      <c r="D87" s="18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="55" t="s">
+        <v>22</v>
+      </c>
+      <c r="B88" s="56" t="s">
+        <v>23</v>
+      </c>
+      <c r="C88" s="56" t="s">
+        <v>24</v>
+      </c>
+      <c r="D88" s="57" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="58" t="s">
+        <v>30</v>
+      </c>
+      <c r="B89" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C89" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D89" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="58"/>
+      <c r="B90" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C90" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D90" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="58"/>
+      <c r="B91" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C91" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D91" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A92" s="58"/>
+      <c r="B92" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C92" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D92" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A93" s="62"/>
+      <c r="B93" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="C93" s="64" t="s">
+        <v>77</v>
+      </c>
+      <c r="D93" s="65" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A94" s="53"/>
+      <c r="B94" s="53"/>
+      <c r="C94" s="53"/>
+      <c r="D94" s="53"/>
+    </row>
+    <row r="95" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="54" t="s">
+        <v>38</v>
+      </c>
+      <c r="B95" s="54"/>
+      <c r="C95" s="54"/>
+      <c r="D95" s="54"/>
+    </row>
+    <row r="96" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A96" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="B96" s="56" t="s">
+        <v>40</v>
+      </c>
+      <c r="C96" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="D96" s="57" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A97" s="66"/>
+      <c r="B97" s="60"/>
+      <c r="C97" s="60"/>
+      <c r="D97" s="61"/>
+    </row>
+    <row r="98" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A98" s="67"/>
+      <c r="B98" s="68"/>
+      <c r="C98" s="68"/>
+      <c r="D98" s="69"/>
+    </row>
+    <row r="99" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A99" s="70"/>
+      <c r="B99" s="71"/>
+      <c r="C99" s="71"/>
+      <c r="D99" s="72"/>
+    </row>
+    <row r="100" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A100" s="73" t="s">
+        <v>43</v>
+      </c>
+      <c r="B100" s="73"/>
+      <c r="C100" s="73"/>
+      <c r="D100" s="73"/>
+    </row>
+    <row r="101" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A101" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="B101" s="56" t="s">
+        <v>44</v>
+      </c>
+      <c r="C101" s="56" t="s">
+        <v>45</v>
+      </c>
+      <c r="D101" s="57" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A102" s="74" t="s">
+        <v>47</v>
+      </c>
+      <c r="B102" s="75" t="s">
+        <v>48</v>
+      </c>
+      <c r="C102" s="76" t="s">
+        <v>56</v>
+      </c>
+      <c r="D102" s="61"/>
+    </row>
+    <row r="103" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A103" s="74" t="s">
+        <v>51</v>
+      </c>
+      <c r="B103" s="75" t="s">
+        <v>52</v>
+      </c>
+      <c r="C103" s="76" t="s">
+        <v>56</v>
+      </c>
+      <c r="D103" s="61"/>
+    </row>
+    <row r="104" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A104" s="74" t="s">
+        <v>54</v>
+      </c>
+      <c r="B104" s="75" t="s">
+        <v>55</v>
+      </c>
+      <c r="C104" s="76" t="s">
+        <v>56</v>
+      </c>
+      <c r="D104" s="61"/>
+    </row>
+    <row r="105" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A105" s="74" t="s">
+        <v>57</v>
+      </c>
+      <c r="B105" s="75" t="s">
+        <v>58</v>
+      </c>
+      <c r="C105" s="76" t="s">
+        <v>56</v>
+      </c>
+      <c r="D105" s="61"/>
+    </row>
+    <row r="106" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A106" s="77" t="s">
+        <v>60</v>
+      </c>
+      <c r="B106" s="78" t="s">
+        <v>61</v>
+      </c>
+      <c r="C106" s="79" t="s">
+        <v>56</v>
+      </c>
+      <c r="D106" s="65"/>
+    </row>
+    <row r="107" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A107" s="53"/>
+      <c r="B107" s="80"/>
+      <c r="C107" s="81"/>
+      <c r="D107" s="81"/>
+    </row>
+    <row r="108" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A108" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="B52" s="86"/>
-      <c r="C52" s="87"/>
-      <c r="D52" s="87"/>
-    </row>
-    <row r="53" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="59" t="s">
+      <c r="B108" s="82"/>
+      <c r="C108" s="83"/>
+      <c r="D108" s="83"/>
+    </row>
+    <row r="109" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A109" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="B53" s="88" t="s">
+      <c r="B109" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="C53" s="89" t="s">
+      <c r="C109" s="85" t="s">
         <v>65</v>
       </c>
-      <c r="D53" s="61" t="s">
+      <c r="D109" s="57" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="70"/>
-      <c r="B54" s="64"/>
-      <c r="C54" s="64"/>
-      <c r="D54" s="65"/>
-    </row>
-    <row r="55" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="90"/>
-      <c r="B55" s="91"/>
-      <c r="C55" s="72"/>
-      <c r="D55" s="73"/>
-    </row>
-    <row r="56" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="74"/>
-      <c r="B56" s="75"/>
-      <c r="C56" s="75"/>
-      <c r="D56" s="76"/>
-    </row>
-    <row r="57" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="1" t="s">
+    <row r="110" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A110" s="66"/>
+      <c r="B110" s="60"/>
+      <c r="C110" s="60"/>
+      <c r="D110" s="61"/>
+    </row>
+    <row r="111" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A111" s="86"/>
+      <c r="B111" s="87"/>
+      <c r="C111" s="68"/>
+      <c r="D111" s="69"/>
+    </row>
+    <row r="112" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A112" s="70"/>
+      <c r="B112" s="71"/>
+      <c r="C112" s="71"/>
+      <c r="D112" s="72"/>
+    </row>
+    <row r="113" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A113" s="105" t="s">
         <v>89</v>
       </c>
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="1"/>
-    </row>
-    <row r="58" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="20"/>
-      <c r="B58" s="20"/>
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
-    </row>
-    <row r="59" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="21" t="s">
+      <c r="B113" s="105"/>
+      <c r="C113" s="105"/>
+      <c r="D113" s="105"/>
+    </row>
+    <row r="114" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A114" s="16"/>
+      <c r="B114" s="16"/>
+      <c r="C114" s="16"/>
+      <c r="D114" s="16"/>
+    </row>
+    <row r="115" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A115" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="B59" s="21"/>
-      <c r="C59" s="21"/>
-      <c r="D59" s="22" t="s">
+      <c r="B115" s="17"/>
+      <c r="C115" s="17"/>
+      <c r="D115" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="23" t="s">
+    <row r="116" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A116" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B60" s="24" t="s">
+      <c r="B116" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C60" s="24" t="s">
+      <c r="C116" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D60" s="25" t="s">
+      <c r="D116" s="21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="26" t="s">
+    <row r="117" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A117" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="B61" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C61" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D61" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="26"/>
-      <c r="B62" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C62" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D62" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="26"/>
-      <c r="B63" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C63" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D63" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="26"/>
-      <c r="B64" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C64" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D64" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="30"/>
-      <c r="B65" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="C65" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="D65" s="33" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="20"/>
-      <c r="B66" s="20"/>
-      <c r="C66" s="20"/>
-      <c r="D66" s="20"/>
-    </row>
-    <row r="67" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="21" t="s">
+      <c r="B117" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C117" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D117" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A118" s="22"/>
+      <c r="B118" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C118" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D118" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A119" s="22"/>
+      <c r="B119" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C119" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D119" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A120" s="22"/>
+      <c r="B120" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C120" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D120" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A121" s="26"/>
+      <c r="B121" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="C121" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D121" s="29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A122" s="16"/>
+      <c r="B122" s="16"/>
+      <c r="C122" s="16"/>
+      <c r="D122" s="16"/>
+    </row>
+    <row r="123" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A123" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B67" s="21"/>
-      <c r="C67" s="21"/>
-      <c r="D67" s="21"/>
-    </row>
-    <row r="68" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="23" t="s">
+      <c r="B123" s="17"/>
+      <c r="C123" s="17"/>
+      <c r="D123" s="17"/>
+    </row>
+    <row r="124" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A124" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B68" s="24" t="s">
+      <c r="B124" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C68" s="24" t="s">
+      <c r="C124" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="D68" s="25" t="s">
+      <c r="D124" s="21" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="35"/>
-      <c r="B69" s="27"/>
-      <c r="C69" s="27"/>
-      <c r="D69" s="28"/>
-    </row>
-    <row r="70" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="39"/>
-      <c r="B70" s="92"/>
-      <c r="C70" s="92"/>
-      <c r="D70" s="93"/>
-    </row>
-    <row r="71" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="94"/>
-      <c r="B71" s="41"/>
-      <c r="C71" s="41"/>
-      <c r="D71" s="95"/>
-    </row>
-    <row r="72" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="42" t="s">
+    <row r="125" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A125" s="31"/>
+      <c r="B125" s="23"/>
+      <c r="C125" s="23"/>
+      <c r="D125" s="24"/>
+    </row>
+    <row r="126" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A126" s="35"/>
+      <c r="B126" s="88"/>
+      <c r="C126" s="88"/>
+      <c r="D126" s="89"/>
+    </row>
+    <row r="127" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A127" s="90"/>
+      <c r="B127" s="37"/>
+      <c r="C127" s="37"/>
+      <c r="D127" s="91"/>
+    </row>
+    <row r="128" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A128" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="B72" s="42"/>
-      <c r="C72" s="42"/>
-      <c r="D72" s="42"/>
-    </row>
-    <row r="73" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="23" t="s">
+      <c r="B128" s="38"/>
+      <c r="C128" s="38"/>
+      <c r="D128" s="38"/>
+    </row>
+    <row r="129" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A129" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B73" s="24" t="s">
+      <c r="B129" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C73" s="24" t="s">
+      <c r="C129" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D73" s="25" t="s">
+      <c r="D129" s="21" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="74" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="43" t="s">
+    <row r="130" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A130" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="B74" s="37" t="s">
+      <c r="B130" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="C74" s="44" t="s">
+      <c r="C130" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D74" s="28"/>
-    </row>
-    <row r="75" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="43" t="s">
+      <c r="D130" s="24"/>
+    </row>
+    <row r="131" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A131" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B75" s="37" t="s">
+      <c r="B131" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="C75" s="44" t="s">
+      <c r="C131" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D75" s="28"/>
-    </row>
-    <row r="76" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="43" t="s">
+      <c r="D131" s="24"/>
+    </row>
+    <row r="132" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A132" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="B76" s="37" t="s">
+      <c r="B132" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="C76" s="44" t="s">
+      <c r="C132" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D76" s="28"/>
-    </row>
-    <row r="77" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="43" t="s">
+      <c r="D132" s="24"/>
+    </row>
+    <row r="133" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A133" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="B77" s="37" t="s">
+      <c r="B133" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="C77" s="44" t="s">
+      <c r="C133" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D77" s="28"/>
-    </row>
-    <row r="78" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="45" t="s">
+      <c r="D133" s="24"/>
+    </row>
+    <row r="134" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A134" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="B78" s="46" t="s">
+      <c r="B134" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="C78" s="47" t="s">
+      <c r="C134" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="D78" s="33"/>
-    </row>
-    <row r="79" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="20"/>
-      <c r="B79" s="48"/>
-      <c r="C79" s="49"/>
-      <c r="D79" s="49"/>
-    </row>
-    <row r="80" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="21" t="s">
+      <c r="D134" s="29"/>
+    </row>
+    <row r="135" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A135" s="16"/>
+      <c r="B135" s="44"/>
+      <c r="C135" s="45"/>
+      <c r="D135" s="45"/>
+    </row>
+    <row r="136" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A136" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B80" s="50"/>
-      <c r="C80" s="51"/>
-      <c r="D80" s="51"/>
-    </row>
-    <row r="81" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="23" t="s">
+      <c r="B136" s="46"/>
+      <c r="C136" s="47"/>
+      <c r="D136" s="47"/>
+    </row>
+    <row r="137" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A137" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B81" s="52" t="s">
+      <c r="B137" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="C81" s="53" t="s">
+      <c r="C137" s="49" t="s">
         <v>65</v>
       </c>
-      <c r="D81" s="25" t="s">
+      <c r="D137" s="21" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="82" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="35"/>
-      <c r="B82" s="27"/>
-      <c r="C82" s="54"/>
-      <c r="D82" s="54"/>
-    </row>
-    <row r="83" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="55"/>
-      <c r="B83" s="96"/>
-      <c r="C83" s="54"/>
-      <c r="D83" s="54"/>
-    </row>
-    <row r="84" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="94"/>
-      <c r="B84" s="41"/>
-      <c r="C84" s="41"/>
-      <c r="D84" s="95"/>
-    </row>
-    <row r="85" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="2" t="s">
+    <row r="138" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A138" s="31"/>
+      <c r="B138" s="23"/>
+      <c r="C138" s="50"/>
+      <c r="D138" s="50"/>
+    </row>
+    <row r="139" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A139" s="51"/>
+      <c r="B139" s="92"/>
+      <c r="C139" s="50"/>
+      <c r="D139" s="50"/>
+    </row>
+    <row r="140" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A140" s="90"/>
+      <c r="B140" s="37"/>
+      <c r="C140" s="37"/>
+      <c r="D140" s="91"/>
+    </row>
+    <row r="141" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A141" s="104" t="s">
         <v>90</v>
       </c>
-      <c r="B85" s="2"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
-    </row>
-    <row r="86" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="57"/>
-      <c r="B86" s="57"/>
-      <c r="C86" s="57"/>
-      <c r="D86" s="57"/>
-    </row>
-    <row r="87" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="58" t="s">
+      <c r="B141" s="104"/>
+      <c r="C141" s="104"/>
+      <c r="D141" s="104"/>
+    </row>
+    <row r="142" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A142" s="53"/>
+      <c r="B142" s="53"/>
+      <c r="C142" s="53"/>
+      <c r="D142" s="53"/>
+    </row>
+    <row r="143" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A143" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="B87" s="58"/>
-      <c r="C87" s="58"/>
-      <c r="D87" s="22" t="s">
+      <c r="B143" s="54"/>
+      <c r="C143" s="54"/>
+      <c r="D143" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="59" t="s">
+    <row r="144" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A144" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="B88" s="60" t="s">
+      <c r="B144" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="C88" s="60" t="s">
+      <c r="C144" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="D88" s="61" t="s">
+      <c r="D144" s="57" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="62" t="s">
+    <row r="145" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A145" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="B89" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C89" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D89" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="62"/>
-      <c r="B90" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C90" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D90" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="62"/>
-      <c r="B91" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C91" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D91" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="62"/>
-      <c r="B92" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C92" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D92" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="66"/>
-      <c r="B93" s="67" t="s">
-        <v>78</v>
-      </c>
-      <c r="C93" s="68" t="s">
-        <v>79</v>
-      </c>
-      <c r="D93" s="69" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="57"/>
-      <c r="B94" s="57"/>
-      <c r="C94" s="57"/>
-      <c r="D94" s="57"/>
-    </row>
-    <row r="95" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="58" t="s">
+      <c r="B145" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C145" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D145" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A146" s="58"/>
+      <c r="B146" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C146" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D146" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A147" s="58"/>
+      <c r="B147" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C147" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D147" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A148" s="58"/>
+      <c r="B148" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C148" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D148" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A149" s="62"/>
+      <c r="B149" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="C149" s="64" t="s">
+        <v>77</v>
+      </c>
+      <c r="D149" s="65" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A150" s="53"/>
+      <c r="B150" s="53"/>
+      <c r="C150" s="53"/>
+      <c r="D150" s="53"/>
+    </row>
+    <row r="151" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A151" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="B95" s="58"/>
-      <c r="C95" s="58"/>
-      <c r="D95" s="58"/>
-    </row>
-    <row r="96" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="59" t="s">
+      <c r="B151" s="54"/>
+      <c r="C151" s="54"/>
+      <c r="D151" s="54"/>
+    </row>
+    <row r="152" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A152" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="B96" s="60" t="s">
+      <c r="B152" s="56" t="s">
         <v>40</v>
       </c>
-      <c r="C96" s="60" t="s">
+      <c r="C152" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="D96" s="61" t="s">
+      <c r="D152" s="57" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="70"/>
-      <c r="B97" s="64"/>
-      <c r="C97" s="64"/>
-      <c r="D97" s="65"/>
-    </row>
-    <row r="98" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="71"/>
-      <c r="B98" s="72"/>
-      <c r="C98" s="72"/>
-      <c r="D98" s="73"/>
-    </row>
-    <row r="99" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="74"/>
-      <c r="B99" s="75"/>
-      <c r="C99" s="75"/>
-      <c r="D99" s="76"/>
-    </row>
-    <row r="100" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="77" t="s">
+    <row r="153" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A153" s="66"/>
+      <c r="B153" s="60"/>
+      <c r="C153" s="60"/>
+      <c r="D153" s="61"/>
+    </row>
+    <row r="154" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A154" s="67"/>
+      <c r="B154" s="68"/>
+      <c r="C154" s="68"/>
+      <c r="D154" s="69"/>
+    </row>
+    <row r="155" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A155" s="70"/>
+      <c r="B155" s="71"/>
+      <c r="C155" s="71"/>
+      <c r="D155" s="72"/>
+    </row>
+    <row r="156" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A156" s="93" t="s">
         <v>43</v>
       </c>
-      <c r="B100" s="77"/>
-      <c r="C100" s="77"/>
-      <c r="D100" s="77"/>
-    </row>
-    <row r="101" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="59" t="s">
+      <c r="B156" s="94"/>
+      <c r="C156" s="94"/>
+      <c r="D156" s="95"/>
+    </row>
+    <row r="157" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A157" s="96" t="s">
         <v>0</v>
       </c>
-      <c r="B101" s="60" t="s">
+      <c r="B157" s="97" t="s">
         <v>44</v>
       </c>
-      <c r="C101" s="60" t="s">
+      <c r="C157" s="97" t="s">
         <v>45</v>
       </c>
-      <c r="D101" s="61" t="s">
+      <c r="D157" s="98" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="102" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="78" t="s">
+    <row r="158" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A158" s="74" t="s">
         <v>47</v>
       </c>
-      <c r="B102" s="79" t="s">
+      <c r="B158" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="C102" s="80" t="s">
+      <c r="C158" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="D102" s="65"/>
-    </row>
-    <row r="103" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A103" s="78" t="s">
+      <c r="D158" s="61"/>
+    </row>
+    <row r="159" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A159" s="74" t="s">
         <v>51</v>
       </c>
-      <c r="B103" s="79" t="s">
+      <c r="B159" s="75" t="s">
         <v>52</v>
       </c>
-      <c r="C103" s="80" t="s">
+      <c r="C159" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="D103" s="65"/>
-    </row>
-    <row r="104" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A104" s="78" t="s">
+      <c r="D159" s="61"/>
+    </row>
+    <row r="160" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A160" s="74" t="s">
         <v>54</v>
       </c>
-      <c r="B104" s="79" t="s">
+      <c r="B160" s="75" t="s">
         <v>55</v>
       </c>
-      <c r="C104" s="80" t="s">
+      <c r="C160" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="D104" s="65"/>
-    </row>
-    <row r="105" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A105" s="78" t="s">
+      <c r="D160" s="61"/>
+    </row>
+    <row r="161" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A161" s="74" t="s">
         <v>57</v>
       </c>
-      <c r="B105" s="79" t="s">
+      <c r="B161" s="75" t="s">
         <v>58</v>
       </c>
-      <c r="C105" s="80" t="s">
+      <c r="C161" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="D105" s="65"/>
-    </row>
-    <row r="106" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A106" s="81" t="s">
+      <c r="D161" s="61"/>
+    </row>
+    <row r="162" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A162" s="77" t="s">
         <v>60</v>
       </c>
-      <c r="B106" s="82" t="s">
+      <c r="B162" s="78" t="s">
         <v>61</v>
       </c>
-      <c r="C106" s="83" t="s">
+      <c r="C162" s="79" t="s">
         <v>56</v>
       </c>
-      <c r="D106" s="69"/>
-    </row>
-    <row r="107" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="57"/>
-      <c r="B107" s="84"/>
-      <c r="C107" s="85"/>
-      <c r="D107" s="85"/>
-    </row>
-    <row r="108" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A108" s="58" t="s">
+      <c r="D162" s="65"/>
+    </row>
+    <row r="163" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A163" s="53"/>
+      <c r="B163" s="80"/>
+      <c r="C163" s="81"/>
+      <c r="D163" s="81"/>
+    </row>
+    <row r="164" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A164" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="B108" s="86"/>
-      <c r="C108" s="87"/>
-      <c r="D108" s="87"/>
-    </row>
-    <row r="109" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="59" t="s">
+      <c r="B164" s="82"/>
+      <c r="C164" s="83"/>
+      <c r="D164" s="83"/>
+    </row>
+    <row r="165" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A165" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="B109" s="88" t="s">
+      <c r="B165" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="C109" s="89" t="s">
+      <c r="C165" s="85" t="s">
         <v>65</v>
       </c>
-      <c r="D109" s="61" t="s">
+      <c r="D165" s="57" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="110" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="70"/>
-      <c r="B110" s="64"/>
-      <c r="C110" s="64"/>
-      <c r="D110" s="65"/>
-    </row>
-    <row r="111" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A111" s="90"/>
-      <c r="B111" s="91"/>
-      <c r="C111" s="72"/>
-      <c r="D111" s="73"/>
-    </row>
-    <row r="112" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" s="74"/>
-      <c r="B112" s="75"/>
-      <c r="C112" s="75"/>
-      <c r="D112" s="76"/>
-    </row>
-    <row r="113" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A113" s="1" t="s">
+    <row r="166" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A166" s="66"/>
+      <c r="B166" s="60"/>
+      <c r="C166" s="60"/>
+      <c r="D166" s="61"/>
+    </row>
+    <row r="167" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A167" s="86"/>
+      <c r="B167" s="87"/>
+      <c r="C167" s="68"/>
+      <c r="D167" s="69"/>
+    </row>
+    <row r="168" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A168" s="70"/>
+      <c r="B168" s="71"/>
+      <c r="C168" s="71"/>
+      <c r="D168" s="72"/>
+    </row>
+    <row r="169" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A169" s="105" t="s">
         <v>91</v>
       </c>
-      <c r="B113" s="1"/>
-      <c r="C113" s="1"/>
-      <c r="D113" s="1"/>
-    </row>
-    <row r="114" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A114" s="20"/>
-      <c r="B114" s="20"/>
-      <c r="C114" s="20"/>
-      <c r="D114" s="20"/>
-    </row>
-    <row r="115" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A115" s="21" t="s">
+      <c r="B169" s="105"/>
+      <c r="C169" s="105"/>
+      <c r="D169" s="105"/>
+    </row>
+    <row r="170" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A170" s="16"/>
+      <c r="B170" s="16"/>
+      <c r="C170" s="16"/>
+      <c r="D170" s="16"/>
+    </row>
+    <row r="171" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A171" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="B115" s="21"/>
-      <c r="C115" s="21"/>
-      <c r="D115" s="22" t="s">
+      <c r="B171" s="17"/>
+      <c r="C171" s="17"/>
+      <c r="D171" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="23" t="s">
+    <row r="172" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A172" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B116" s="24" t="s">
+      <c r="B172" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C116" s="24" t="s">
+      <c r="C172" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D116" s="25" t="s">
+      <c r="D172" s="21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="117" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A117" s="26" t="s">
+    <row r="173" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A173" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="B117" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C117" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D117" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A118" s="26"/>
-      <c r="B118" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C118" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D118" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="26"/>
-      <c r="B119" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C119" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D119" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A120" s="26"/>
-      <c r="B120" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C120" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D120" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A121" s="30"/>
-      <c r="B121" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="C121" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="D121" s="33" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A122" s="20"/>
-      <c r="B122" s="20"/>
-      <c r="C122" s="20"/>
-      <c r="D122" s="20"/>
-    </row>
-    <row r="123" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A123" s="21" t="s">
+      <c r="B173" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C173" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D173" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A174" s="22"/>
+      <c r="B174" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C174" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D174" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A175" s="22"/>
+      <c r="B175" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C175" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D175" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A176" s="22"/>
+      <c r="B176" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C176" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D176" s="24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A177" s="26"/>
+      <c r="B177" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="C177" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D177" s="29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A178" s="16"/>
+      <c r="B178" s="16"/>
+      <c r="C178" s="16"/>
+      <c r="D178" s="16"/>
+    </row>
+    <row r="179" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A179" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B123" s="21"/>
-      <c r="C123" s="21"/>
-      <c r="D123" s="21"/>
-    </row>
-    <row r="124" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="23" t="s">
+      <c r="B179" s="17"/>
+      <c r="C179" s="17"/>
+      <c r="D179" s="17"/>
+    </row>
+    <row r="180" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A180" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B124" s="24" t="s">
+      <c r="B180" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C124" s="24" t="s">
+      <c r="C180" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="D124" s="25" t="s">
+      <c r="D180" s="21" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="35"/>
-      <c r="B125" s="27"/>
-      <c r="C125" s="27"/>
-      <c r="D125" s="28"/>
-    </row>
-    <row r="126" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A126" s="39"/>
-      <c r="B126" s="92"/>
-      <c r="C126" s="92"/>
-      <c r="D126" s="93"/>
-    </row>
-    <row r="127" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="94"/>
-      <c r="B127" s="41"/>
-      <c r="C127" s="41"/>
-      <c r="D127" s="95"/>
-    </row>
-    <row r="128" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="42" t="s">
+    <row r="181" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A181" s="31"/>
+      <c r="B181" s="23"/>
+      <c r="C181" s="23"/>
+      <c r="D181" s="24"/>
+    </row>
+    <row r="182" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A182" s="35"/>
+      <c r="B182" s="88"/>
+      <c r="C182" s="88"/>
+      <c r="D182" s="89"/>
+    </row>
+    <row r="183" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A183" s="90"/>
+      <c r="B183" s="37"/>
+      <c r="C183" s="37"/>
+      <c r="D183" s="91"/>
+    </row>
+    <row r="184" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A184" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="B128" s="42"/>
-      <c r="C128" s="42"/>
-      <c r="D128" s="42"/>
-    </row>
-    <row r="129" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="23" t="s">
+      <c r="B184" s="38"/>
+      <c r="C184" s="38"/>
+      <c r="D184" s="38"/>
+    </row>
+    <row r="185" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A185" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B129" s="24" t="s">
+      <c r="B185" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C129" s="24" t="s">
+      <c r="C185" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D129" s="25" t="s">
+      <c r="D185" s="21" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="130" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A130" s="43" t="s">
+    <row r="186" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A186" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="B130" s="37" t="s">
+      <c r="B186" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="C130" s="44" t="s">
+      <c r="C186" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D130" s="28"/>
-    </row>
-    <row r="131" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A131" s="43" t="s">
+      <c r="D186" s="24"/>
+    </row>
+    <row r="187" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A187" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B131" s="37" t="s">
+      <c r="B187" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="C131" s="44" t="s">
+      <c r="C187" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D131" s="28"/>
-    </row>
-    <row r="132" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="43" t="s">
+      <c r="D187" s="24"/>
+    </row>
+    <row r="188" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A188" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="B132" s="37" t="s">
+      <c r="B188" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="C132" s="44" t="s">
+      <c r="C188" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D132" s="28"/>
-    </row>
-    <row r="133" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="43" t="s">
+      <c r="D188" s="24"/>
+    </row>
+    <row r="189" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A189" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="B133" s="37" t="s">
+      <c r="B189" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="C133" s="44" t="s">
+      <c r="C189" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D133" s="28"/>
-    </row>
-    <row r="134" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="45" t="s">
+      <c r="D189" s="24"/>
+    </row>
+    <row r="190" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A190" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="B134" s="46" t="s">
+      <c r="B190" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="C134" s="47" t="s">
+      <c r="C190" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="D134" s="33"/>
-    </row>
-    <row r="135" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A135" s="20"/>
-      <c r="B135" s="48"/>
-      <c r="C135" s="49"/>
-      <c r="D135" s="49"/>
-    </row>
-    <row r="136" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A136" s="21" t="s">
+      <c r="D190" s="29"/>
+    </row>
+    <row r="191" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A191" s="16"/>
+      <c r="B191" s="44"/>
+      <c r="C191" s="45"/>
+      <c r="D191" s="45"/>
+    </row>
+    <row r="192" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A192" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B136" s="50"/>
-      <c r="C136" s="51"/>
-      <c r="D136" s="51"/>
-    </row>
-    <row r="137" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A137" s="23" t="s">
+      <c r="B192" s="46"/>
+      <c r="C192" s="47"/>
+      <c r="D192" s="47"/>
+    </row>
+    <row r="193" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A193" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B137" s="52" t="s">
+      <c r="B193" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="C137" s="53" t="s">
+      <c r="C193" s="49" t="s">
         <v>65</v>
       </c>
-      <c r="D137" s="25" t="s">
+      <c r="D193" s="21" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="35"/>
-      <c r="B138" s="27"/>
-      <c r="C138" s="54"/>
-      <c r="D138" s="54"/>
-    </row>
-    <row r="139" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A139" s="55"/>
-      <c r="B139" s="96"/>
-      <c r="C139" s="54"/>
-      <c r="D139" s="54"/>
-    </row>
-    <row r="140" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="94"/>
-      <c r="B140" s="41"/>
-      <c r="C140" s="41"/>
-      <c r="D140" s="95"/>
-    </row>
-    <row r="141" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="2" t="s">
+    <row r="194" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A194" s="31"/>
+      <c r="B194" s="23"/>
+      <c r="C194" s="50"/>
+      <c r="D194" s="50"/>
+    </row>
+    <row r="195" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A195" s="51"/>
+      <c r="B195" s="92"/>
+      <c r="C195" s="50"/>
+      <c r="D195" s="50"/>
+    </row>
+    <row r="196" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A196" s="90"/>
+      <c r="B196" s="37"/>
+      <c r="C196" s="37"/>
+      <c r="D196" s="91"/>
+    </row>
+    <row r="197" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A197" s="104" t="s">
         <v>92</v>
       </c>
-      <c r="B141" s="2"/>
-      <c r="C141" s="2"/>
-      <c r="D141" s="2"/>
-    </row>
-    <row r="142" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A142" s="57"/>
-      <c r="B142" s="57"/>
-      <c r="C142" s="57"/>
-      <c r="D142" s="57"/>
-    </row>
-    <row r="143" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A143" s="58" t="s">
+      <c r="B197" s="104"/>
+      <c r="C197" s="104"/>
+      <c r="D197" s="104"/>
+    </row>
+    <row r="198" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A198" s="53"/>
+      <c r="B198" s="53"/>
+      <c r="C198" s="53"/>
+      <c r="D198" s="53"/>
+    </row>
+    <row r="199" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A199" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="B143" s="58"/>
-      <c r="C143" s="58"/>
-      <c r="D143" s="22" t="s">
+      <c r="B199" s="54"/>
+      <c r="C199" s="54"/>
+      <c r="D199" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="59" t="s">
+    <row r="200" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A200" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="B144" s="60" t="s">
+      <c r="B200" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="C144" s="60" t="s">
+      <c r="C200" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="D144" s="61" t="s">
+      <c r="D200" s="57" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="145" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="62" t="s">
+    <row r="201" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A201" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="B145" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C145" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D145" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="146" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="62"/>
-      <c r="B146" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C146" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D146" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="147" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="62"/>
-      <c r="B147" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C147" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D147" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="62"/>
-      <c r="B148" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C148" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D148" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="66"/>
-      <c r="B149" s="67" t="s">
-        <v>78</v>
-      </c>
-      <c r="C149" s="68" t="s">
-        <v>79</v>
-      </c>
-      <c r="D149" s="69" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A150" s="57"/>
-      <c r="B150" s="57"/>
-      <c r="C150" s="57"/>
-      <c r="D150" s="57"/>
-    </row>
-    <row r="151" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="58" t="s">
+      <c r="B201" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C201" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D201" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A202" s="58"/>
+      <c r="B202" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C202" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D202" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A203" s="58"/>
+      <c r="B203" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C203" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D203" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A204" s="58"/>
+      <c r="B204" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C204" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D204" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A205" s="62"/>
+      <c r="B205" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="C205" s="64" t="s">
+        <v>77</v>
+      </c>
+      <c r="D205" s="65" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A206" s="53"/>
+      <c r="B206" s="53"/>
+      <c r="C206" s="53"/>
+      <c r="D206" s="53"/>
+    </row>
+    <row r="207" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A207" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="B151" s="58"/>
-      <c r="C151" s="58"/>
-      <c r="D151" s="58"/>
-    </row>
-    <row r="152" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="59" t="s">
+      <c r="B207" s="54"/>
+      <c r="C207" s="54"/>
+      <c r="D207" s="54"/>
+    </row>
+    <row r="208" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A208" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="B152" s="60" t="s">
+      <c r="B208" s="56" t="s">
         <v>40</v>
       </c>
-      <c r="C152" s="60" t="s">
+      <c r="C208" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="D152" s="61" t="s">
+      <c r="D208" s="57" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="153" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="70"/>
-      <c r="B153" s="64"/>
-      <c r="C153" s="64"/>
-      <c r="D153" s="65"/>
-    </row>
-    <row r="154" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="71"/>
-      <c r="B154" s="72"/>
-      <c r="C154" s="72"/>
-      <c r="D154" s="73"/>
-    </row>
-    <row r="155" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="74"/>
-      <c r="B155" s="75"/>
-      <c r="C155" s="75"/>
-      <c r="D155" s="76"/>
-    </row>
-    <row r="156" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="97" t="s">
+    <row r="209" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A209" s="66"/>
+      <c r="B209" s="60"/>
+      <c r="C209" s="60"/>
+      <c r="D209" s="61"/>
+    </row>
+    <row r="210" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A210" s="67"/>
+      <c r="B210" s="68"/>
+      <c r="C210" s="68"/>
+      <c r="D210" s="69"/>
+    </row>
+    <row r="211" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A211" s="70"/>
+      <c r="B211" s="71"/>
+      <c r="C211" s="71"/>
+      <c r="D211" s="72"/>
+    </row>
+    <row r="212" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A212" s="73" t="s">
         <v>43</v>
       </c>
-      <c r="B156" s="98"/>
-      <c r="C156" s="98"/>
-      <c r="D156" s="99"/>
-    </row>
-    <row r="157" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A157" s="100" t="s">
+      <c r="B212" s="73"/>
+      <c r="C212" s="73"/>
+      <c r="D212" s="73"/>
+    </row>
+    <row r="213" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A213" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B157" s="101" t="s">
+      <c r="B213" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="C157" s="101" t="s">
+      <c r="C213" s="56" t="s">
         <v>45</v>
       </c>
-      <c r="D157" s="102" t="s">
+      <c r="D213" s="57" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="158" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="78" t="s">
+    <row r="214" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A214" s="74" t="s">
         <v>47</v>
       </c>
-      <c r="B158" s="79" t="s">
+      <c r="B214" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="C158" s="80" t="s">
+      <c r="C214" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="D158" s="65"/>
-    </row>
-    <row r="159" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="78" t="s">
+      <c r="D214" s="61"/>
+    </row>
+    <row r="215" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A215" s="74" t="s">
         <v>51</v>
       </c>
-      <c r="B159" s="79" t="s">
+      <c r="B215" s="75" t="s">
         <v>52</v>
       </c>
-      <c r="C159" s="80" t="s">
+      <c r="C215" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="D159" s="65"/>
-    </row>
-    <row r="160" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="78" t="s">
+      <c r="D215" s="61"/>
+    </row>
+    <row r="216" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A216" s="74" t="s">
         <v>54</v>
       </c>
-      <c r="B160" s="79" t="s">
+      <c r="B216" s="75" t="s">
         <v>55</v>
       </c>
-      <c r="C160" s="80" t="s">
+      <c r="C216" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="D160" s="65"/>
-    </row>
-    <row r="161" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A161" s="78" t="s">
+      <c r="D216" s="61"/>
+    </row>
+    <row r="217" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A217" s="74" t="s">
         <v>57</v>
       </c>
-      <c r="B161" s="79" t="s">
+      <c r="B217" s="75" t="s">
         <v>58</v>
       </c>
-      <c r="C161" s="80" t="s">
+      <c r="C217" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="D161" s="65"/>
-    </row>
-    <row r="162" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A162" s="81" t="s">
+      <c r="D217" s="61"/>
+    </row>
+    <row r="218" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A218" s="77" t="s">
         <v>60</v>
       </c>
-      <c r="B162" s="82" t="s">
+      <c r="B218" s="78" t="s">
         <v>61</v>
       </c>
-      <c r="C162" s="83" t="s">
+      <c r="C218" s="79" t="s">
         <v>56</v>
       </c>
-      <c r="D162" s="69"/>
-    </row>
-    <row r="163" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="57"/>
-      <c r="B163" s="84"/>
-      <c r="C163" s="85"/>
-      <c r="D163" s="85"/>
-    </row>
-    <row r="164" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="58" t="s">
+      <c r="D218" s="65"/>
+    </row>
+    <row r="219" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A219" s="53"/>
+      <c r="B219" s="80"/>
+      <c r="C219" s="81"/>
+      <c r="D219" s="81"/>
+    </row>
+    <row r="220" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A220" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="B164" s="86"/>
-      <c r="C164" s="87"/>
-      <c r="D164" s="87"/>
-    </row>
-    <row r="165" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A165" s="59" t="s">
+      <c r="B220" s="82"/>
+      <c r="C220" s="83"/>
+      <c r="D220" s="83"/>
+    </row>
+    <row r="221" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A221" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="B165" s="88" t="s">
+      <c r="B221" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="C165" s="89" t="s">
+      <c r="C221" s="85" t="s">
         <v>65</v>
       </c>
-      <c r="D165" s="61" t="s">
+      <c r="D221" s="57" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="166" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A166" s="70"/>
-      <c r="B166" s="64"/>
-      <c r="C166" s="64"/>
-      <c r="D166" s="65"/>
-    </row>
-    <row r="167" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A167" s="90"/>
-      <c r="B167" s="91"/>
-      <c r="C167" s="72"/>
-      <c r="D167" s="73"/>
-    </row>
-    <row r="168" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A168" s="74"/>
-      <c r="B168" s="75"/>
-      <c r="C168" s="75"/>
-      <c r="D168" s="76"/>
-    </row>
-    <row r="169" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A169" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B169" s="1"/>
-      <c r="C169" s="1"/>
-      <c r="D169" s="1"/>
-    </row>
-    <row r="170" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A170" s="20"/>
-      <c r="B170" s="20"/>
-      <c r="C170" s="20"/>
-      <c r="D170" s="20"/>
-    </row>
-    <row r="171" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A171" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="B171" s="21"/>
-      <c r="C171" s="21"/>
-      <c r="D171" s="22" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="172" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A172" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B172" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="C172" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="D172" s="25" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="173" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A173" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="B173" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C173" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D173" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A174" s="26"/>
-      <c r="B174" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C174" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D174" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="175" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A175" s="26"/>
-      <c r="B175" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C175" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D175" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="176" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A176" s="26"/>
-      <c r="B176" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C176" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D176" s="28" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A177" s="30"/>
-      <c r="B177" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="C177" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="D177" s="33" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A178" s="20"/>
-      <c r="B178" s="20"/>
-      <c r="C178" s="20"/>
-      <c r="D178" s="20"/>
-    </row>
-    <row r="179" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A179" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="B179" s="21"/>
-      <c r="C179" s="21"/>
-      <c r="D179" s="21"/>
-    </row>
-    <row r="180" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A180" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="B180" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C180" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="D180" s="25" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A181" s="35"/>
-      <c r="B181" s="27"/>
-      <c r="C181" s="27"/>
-      <c r="D181" s="28"/>
-    </row>
-    <row r="182" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A182" s="39"/>
-      <c r="B182" s="92"/>
-      <c r="C182" s="92"/>
-      <c r="D182" s="93"/>
-    </row>
-    <row r="183" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A183" s="94"/>
-      <c r="B183" s="41"/>
-      <c r="C183" s="41"/>
-      <c r="D183" s="95"/>
-    </row>
-    <row r="184" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A184" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="B184" s="42"/>
-      <c r="C184" s="42"/>
-      <c r="D184" s="42"/>
-    </row>
-    <row r="185" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A185" s="23" t="s">
-        <v>0</v>
-      </c>
-      <c r="B185" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="C185" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="D185" s="25" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="186" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A186" s="43" t="s">
-        <v>47</v>
-      </c>
-      <c r="B186" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="C186" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="D186" s="28"/>
-    </row>
-    <row r="187" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A187" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="B187" s="37" t="s">
-        <v>52</v>
-      </c>
-      <c r="C187" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="D187" s="28"/>
-    </row>
-    <row r="188" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A188" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="B188" s="37" t="s">
-        <v>55</v>
-      </c>
-      <c r="C188" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="D188" s="28"/>
-    </row>
-    <row r="189" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A189" s="43" t="s">
-        <v>57</v>
-      </c>
-      <c r="B189" s="37" t="s">
-        <v>58</v>
-      </c>
-      <c r="C189" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="D189" s="28"/>
-    </row>
-    <row r="190" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A190" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="B190" s="46" t="s">
-        <v>61</v>
-      </c>
-      <c r="C190" s="47" t="s">
-        <v>56</v>
-      </c>
-      <c r="D190" s="33"/>
-    </row>
-    <row r="191" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A191" s="20"/>
-      <c r="B191" s="48"/>
-      <c r="C191" s="49"/>
-      <c r="D191" s="49"/>
-    </row>
-    <row r="192" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A192" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="B192" s="50"/>
-      <c r="C192" s="51"/>
-      <c r="D192" s="51"/>
-    </row>
-    <row r="193" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A193" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="B193" s="52" t="s">
-        <v>64</v>
-      </c>
-      <c r="C193" s="53" t="s">
-        <v>65</v>
-      </c>
-      <c r="D193" s="25" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="194" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A194" s="35"/>
-      <c r="B194" s="27"/>
-      <c r="C194" s="54"/>
-      <c r="D194" s="54"/>
-    </row>
-    <row r="195" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A195" s="55"/>
-      <c r="B195" s="96"/>
-      <c r="C195" s="54"/>
-      <c r="D195" s="54"/>
-    </row>
-    <row r="196" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A196" s="94"/>
-      <c r="B196" s="41"/>
-      <c r="C196" s="41"/>
-      <c r="D196" s="95"/>
-    </row>
-    <row r="197" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A197" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B197" s="2"/>
-      <c r="C197" s="2"/>
-      <c r="D197" s="2"/>
-    </row>
-    <row r="198" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A198" s="57"/>
-      <c r="B198" s="57"/>
-      <c r="C198" s="57"/>
-      <c r="D198" s="57"/>
-    </row>
-    <row r="199" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A199" s="58" t="s">
-        <v>68</v>
-      </c>
-      <c r="B199" s="58"/>
-      <c r="C199" s="58"/>
-      <c r="D199" s="22" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="200" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A200" s="59" t="s">
-        <v>22</v>
-      </c>
-      <c r="B200" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="C200" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="D200" s="61" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="201" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A201" s="62" t="s">
-        <v>30</v>
-      </c>
-      <c r="B201" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C201" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D201" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="202" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A202" s="62"/>
-      <c r="B202" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C202" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D202" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="203" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A203" s="62"/>
-      <c r="B203" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C203" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D203" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="204" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A204" s="62"/>
-      <c r="B204" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C204" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D204" s="65" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="205" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A205" s="66"/>
-      <c r="B205" s="67" t="s">
-        <v>78</v>
-      </c>
-      <c r="C205" s="68" t="s">
-        <v>79</v>
-      </c>
-      <c r="D205" s="69" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="206" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A206" s="57"/>
-      <c r="B206" s="57"/>
-      <c r="C206" s="57"/>
-      <c r="D206" s="57"/>
-    </row>
-    <row r="207" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A207" s="58" t="s">
-        <v>38</v>
-      </c>
-      <c r="B207" s="58"/>
-      <c r="C207" s="58"/>
-      <c r="D207" s="58"/>
-    </row>
-    <row r="208" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A208" s="59" t="s">
-        <v>39</v>
-      </c>
-      <c r="B208" s="60" t="s">
-        <v>40</v>
-      </c>
-      <c r="C208" s="60" t="s">
-        <v>41</v>
-      </c>
-      <c r="D208" s="61" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="209" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A209" s="70"/>
-      <c r="B209" s="64"/>
-      <c r="C209" s="64"/>
-      <c r="D209" s="65"/>
-    </row>
-    <row r="210" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A210" s="71"/>
-      <c r="B210" s="72"/>
-      <c r="C210" s="72"/>
-      <c r="D210" s="73"/>
-    </row>
-    <row r="211" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A211" s="74"/>
-      <c r="B211" s="75"/>
-      <c r="C211" s="75"/>
-      <c r="D211" s="76"/>
-    </row>
-    <row r="212" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A212" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="B212" s="77"/>
-      <c r="C212" s="77"/>
-      <c r="D212" s="77"/>
-    </row>
-    <row r="213" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A213" s="59" t="s">
-        <v>0</v>
-      </c>
-      <c r="B213" s="60" t="s">
-        <v>44</v>
-      </c>
-      <c r="C213" s="60" t="s">
-        <v>45</v>
-      </c>
-      <c r="D213" s="61" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="214" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A214" s="78" t="s">
-        <v>47</v>
-      </c>
-      <c r="B214" s="79" t="s">
-        <v>48</v>
-      </c>
-      <c r="C214" s="80" t="s">
-        <v>56</v>
-      </c>
-      <c r="D214" s="65"/>
-    </row>
-    <row r="215" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A215" s="78" t="s">
-        <v>51</v>
-      </c>
-      <c r="B215" s="79" t="s">
-        <v>52</v>
-      </c>
-      <c r="C215" s="80" t="s">
-        <v>56</v>
-      </c>
-      <c r="D215" s="65"/>
-    </row>
-    <row r="216" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A216" s="78" t="s">
-        <v>54</v>
-      </c>
-      <c r="B216" s="79" t="s">
-        <v>55</v>
-      </c>
-      <c r="C216" s="80" t="s">
-        <v>56</v>
-      </c>
-      <c r="D216" s="65"/>
-    </row>
-    <row r="217" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A217" s="78" t="s">
-        <v>57</v>
-      </c>
-      <c r="B217" s="79" t="s">
-        <v>58</v>
-      </c>
-      <c r="C217" s="80" t="s">
-        <v>56</v>
-      </c>
-      <c r="D217" s="65"/>
-    </row>
-    <row r="218" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A218" s="81" t="s">
-        <v>60</v>
-      </c>
-      <c r="B218" s="82" t="s">
-        <v>61</v>
-      </c>
-      <c r="C218" s="83" t="s">
-        <v>56</v>
-      </c>
-      <c r="D218" s="69"/>
-    </row>
-    <row r="219" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A219" s="57"/>
-      <c r="B219" s="84"/>
-      <c r="C219" s="85"/>
-      <c r="D219" s="85"/>
-    </row>
-    <row r="220" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A220" s="58" t="s">
-        <v>63</v>
-      </c>
-      <c r="B220" s="86"/>
-      <c r="C220" s="87"/>
-      <c r="D220" s="87"/>
-    </row>
-    <row r="221" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A221" s="59" t="s">
-        <v>39</v>
-      </c>
-      <c r="B221" s="88" t="s">
-        <v>64</v>
-      </c>
-      <c r="C221" s="89" t="s">
-        <v>65</v>
-      </c>
-      <c r="D221" s="61" t="s">
-        <v>66</v>
-      </c>
-    </row>
     <row r="222" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A222" s="71"/>
-      <c r="B222" s="72"/>
-      <c r="C222" s="103"/>
-      <c r="D222" s="104"/>
+      <c r="A222" s="67"/>
+      <c r="B222" s="68"/>
+      <c r="C222" s="99"/>
+      <c r="D222" s="100"/>
     </row>
     <row r="223" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A223" s="105"/>
-      <c r="B223" s="105"/>
-      <c r="C223" s="105"/>
-      <c r="D223" s="105"/>
+      <c r="A223" s="101"/>
+      <c r="B223" s="101"/>
+      <c r="C223" s="101"/>
+      <c r="D223" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -4572,7 +4572,7 @@
     </row>
     <row r="2" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Update portfolio lessons and official logbook
</commit_message>
<xml_diff>
--- a/public/Integraal_Sprint_Logboek_Officieel.xlsx
+++ b/public/Integraal_Sprint_Logboek_Officieel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasmijnmesu/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasmijnmesu/Desktop/Mijn Projecten/Portfolio-Jasmijn-Mesu/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5AE274C6-02B1-D24C-9FDD-BC962E88A980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E2A49F-CA74-6848-B436-A938A14A20AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10500" yWindow="760" windowWidth="18900" windowHeight="17320" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17360" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -30,15 +30,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="111">
   <si>
     <t>LU</t>
   </si>
@@ -266,6 +263,33 @@
     <t>Wat ga je anders doen?</t>
   </si>
   <si>
+    <t>Websites zoals NEN Connect bevatten veel juridische regels. Daardoor bleek mijn idee niet haalbaar. Na sparren met Jan heb ik het losgelaten. Ik heb geleerd dat je soms hele leuke ideeën hebt, maar dat je sommige dingen moet loslaten omdat ze niet haalbaar zijn.</t>
+  </si>
+  <si>
+    <t>Sparren met mijn coach over mijn ideeën en kritisch blijven op wat bronnen en AI voorstellen.</t>
+  </si>
+  <si>
+    <t>Bij een nieuw idee eerst de haalbaarheid uitzoeken (juridisch en welke informatie ik mag gebruiken), voordat ik veel tijd in het uitwerken steek. Een idee sneller loslaten als het niet kan.</t>
+  </si>
+  <si>
+    <t>Ik heb via Jan contact opgenomen met Dotslash om meer uit mijn minor te halen en te vragen naar een opdracht. Ik heb geleerd dat je moet durven vragen.</t>
+  </si>
+  <si>
+    <t>Zelf contact zoeken en vragen stellen.</t>
+  </si>
+  <si>
+    <t>Eerder en vaker zelf vragen stellen aan coaches en organisaties, in plaats van te wachten op een opdracht.</t>
+  </si>
+  <si>
+    <t>AI wordt in mijn beroep steeds belangrijker en iedereen moet het leren. Het fysieke contact met mensen blijft belangrijk en wordt misschien nog belangrijker.</t>
+  </si>
+  <si>
+    <t>AI gebruiken als assistent en niet als vervanging, en bewust kiezen welke tool bij welke taak past.</t>
+  </si>
+  <si>
+    <t>Naast AI-vaardigheden ook blijven ontwikkelen wat AI niet kan overnemen, zoals samenwerken en persoonlijk contact.</t>
+  </si>
+  <si>
     <t>SPRINT 2</t>
   </si>
   <si>
@@ -277,6 +301,11 @@
 zodat ik kan onderbouwen of en hoe een agentic aanpak waarde toevoegt aan mijn specifieke minoroplossing.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. DataCamp-cursus "Introduction to AI Agents" succesvol afgerond, inclusief certificaat/bewijs van afronding in logboek.
+2. Een geschreven samenvatting waar de stof besproken wordt en je ten alle tijden de stof terug kan vinden
+3. De samenvatting is toegevoegd aan mijn portfolio om deze altijd bij de hand te hebben. </t>
+  </si>
+  <si>
     <t>1. Betrouwbaarheid &amp; herkomst: gebruik van actuele, gereputeerde bronnen en correcte bronvermelding.
 2. Diepgang &amp; onderbouwing: helder onderscheid gemaakt tussen eenvoudige prompt-chains/workflows en daadwerkelijke autonome agents.
 3. Toepasbaarheid: de vertaalslag sluit direct aan op de context van het eigen projectportfolio.</t>
@@ -285,6 +314,11 @@
     <t>Als AI-projectmanager in opleiding,
 wil ik de bedrijfsactiviteiten, laadinfrastructuur-diensten en potentiële AI-kansen van Blue Current onderzoeken,
 zodat ik tijdens het eerste intakegesprek direct gerichte AI-use cases kan pitchen en een scherpe minoropdracht kan formuleren (Leeruitkomst: Impact &amp; Oplossing).</t>
+  </si>
+  <si>
+    <t>1. Een compact onderzoeksverslag met daarin de kernactiviteiten en propositie van Blue Current, en de huidige technologie- en laadinfrastructuurcontext.
+2. Minimaal 3 concrete AI-kansen/use cases uitgewerkt (bijv. slim laden/netcongestie, voorspellend onderhoud, geautomatiseerde support).
+3. Een gestructureerde vragenlijst (5–8 vragen) voor het intakegesprek met Blue Current.</t>
   </si>
   <si>
     <t>1. Bronnen &amp; herkomst: relevante openbare bronnen gebruikt (website, nieuws, LinkedIn) met expliciete bronvermelding.
@@ -309,6 +343,54 @@
 3. De opzet en code van de website zijn netjes gestructureerd en onderhoudbaar voor verdere uitbreiding in Sprint 3.</t>
   </si>
   <si>
+    <t xml:space="preserve">Shahmeer </t>
+  </si>
+  <si>
+    <t>Zoek uit wat je daarvoor kan doen met AI. Stuur nog een mail naar Norm. Leer je basis via datacamp. Onderzoek of de website echt nodig is om te verbeteren</t>
+  </si>
+  <si>
+    <t>Op advies ga ik een mail sturen en kijken of ik reactie kan ontvangen. Verder zorg ik dat ik mij nog meer ga verdiepen door middel van Datacamp</t>
+  </si>
+  <si>
+    <t>Ronald Boiten</t>
+  </si>
+  <si>
+    <t>Ik vind het fijn dat mijn werk nu veel duidelijker naar voren komt.De fotografie mag inderdaad groter, maar niet te gelikt. Hou de teksten kort. Ik wil wel mijn hele oeuvre kunnen blijven tonen.De typografie moet echt kloppen.</t>
+  </si>
+  <si>
+    <t>In de volgende sprint staat gebruikersvalidatie centraal. Ik test de eerste redesign met de eigenaar, verwerk feedback op visuele identiteit, content en gebruikservaring en werk de homepage responsive en inhoudelijk correct uit. Pas na goedkeuring van de visuele frontend start ik met de technische beheeromgeving en backend.</t>
+  </si>
+  <si>
+    <t>In Sprint 2 leverde ik het eerste werkende prototype van mijn vernieuwde portfoliowebsite op en presenteerde ik dit, samen met de gebruikte AI-systemen, aan Ronald Boiten. Ik liet zien hoe zijn grafische stijl en kleurgebruik in het ontwerp waren verwerkt en welke AI-tools ik daarvoor had ingezet. Ronald gaf concrete feedback op de fotografie, de teksten en de typografie, die ik direct heb vertaald naar aanpassingen voor Sprint 3. Daarmee heb ik niet alleen een praktijkgerichte AI-oplossing gerealiseerd, maar deze ook daadwerkelijk gepresenteerd aan een echte opdrachtgever en verwerkt in een concreet vervolgplan.</t>
+  </si>
+  <si>
+    <t>Ook in Sprint 2 koos ik per taak een andere tool. Voor de Learning Story rondom AI-agents volgde ik de DataCamp-cursus "Introduction to AI Agents" en vergeleek ik een agentic aanpak met mijn huidige werkwijze. Voor het onderzoek naar Blue Current combineerde ik deskresearch met een LLM om gerichte AI-kansen te formuleren voor het intakegesprek. Voor het prototype van de portfoliowebsite gebruikte ik opnieuw Visual Studio Code, GitHub en Vercel om de website live te zetten, en liet ik het resultaat beoordelen door Ronald Boiten. Zo zette ik per onderdeel bewust de tool in die het beste bij de taak paste.</t>
+  </si>
+  <si>
+    <t>Ik stuurde Sprint 2 grotendeels zelf aan. Ik koos zelf de DataCamp-cursus om mijn kennis over AI-agents te verdiepen, plande zelf het onderzoek naar Blue Current en de bijbehorende vragenlijst, en regelde zelfstandig de afspraak met Ronald Boiten om het prototype te bespreken. Na de feedback van Shahmeer en Ronald bepaalde ik zelf mijn vervolgstappen: eerst gebruikersvalidatie van het ontwerp, daarna pas de technische beheeromgeving. Ik hield dus zelf overzicht over mijn planning en stuurde bij op basis van de feedback die ik kreeg, zonder dat iemand mij een vast stappenplan gaf.</t>
+  </si>
+  <si>
+    <t>AI-agents zijn heel belangrijk en er valt heel veel over te leren. Ik heb de basis geleerd via DataCamp, maar ik heb het idee dat ik er nog lang niet alles uit heb gehaald.</t>
+  </si>
+  <si>
+    <t>Eerst de basis leren via een cursus (DataCamp) voordat ik iets ga bouwen.</t>
+  </si>
+  <si>
+    <t>Mij verder verdiepen in AI-agents en uitzoeken wat ik in mijn eigen opdracht kan gebruiken. De keuze voor een agent-aanpak onderbouwen met een aparte Research Story.</t>
+  </si>
+  <si>
+    <t>Het is belangrijk om goed contact te onderhouden met je opdrachtgever en hem mee te nemen in alle stappen. Zo krijg je het mooiste resultaat. De feedback van Ronald op de fotografie, de teksten en de typografie maakte mijn ontwerp beter.</t>
+  </si>
+  <si>
+    <t>Mijn opdrachtgever bij elke stap betrekken, zijn feedback vastleggen en het ontwerp laten beoordelen voordat ik de technische kant bouw.</t>
+  </si>
+  <si>
+    <t>Eerder en vaker afstemmen met Ronald, zodat verbeterpunten eerder zichtbaar zijn.</t>
+  </si>
+  <si>
+    <t>SPRINT 3</t>
+  </si>
+  <si>
     <t>Als &lt; &gt; ,wil ik &lt; &gt; ,zodat &lt; &gt;</t>
   </si>
   <si>
@@ -317,36 +399,6 @@
 3. </t>
   </si>
   <si>
-    <t xml:space="preserve">Shahmeer </t>
-  </si>
-  <si>
-    <t>Zoek uit wat je daarvoor kan doen met AI. Stuur nog een mail naar Norm. Leer je basis via datacamp. Onderzoek of de website echt nodig is om te verbeteren</t>
-  </si>
-  <si>
-    <t>Op advies ga ik een mail sturen en kijken of ik reactie kan ontvangen. Verder zorg ik dat ik mij nog meer ga verdiepen door middel van Datacamp</t>
-  </si>
-  <si>
-    <t>Ronald Boiten</t>
-  </si>
-  <si>
-    <t>Ik vind het fijn dat mijn werk nu veel duidelijker naar voren komt.De fotografie mag inderdaad groter, maar niet te gelikt. Hou de teksten kort. Ik wil wel mijn hele oeuvre kunnen blijven tonen.De typografie moet echt kloppen.</t>
-  </si>
-  <si>
-    <t>In de volgende sprint staat gebruikersvalidatie centraal. Ik test de eerste redesign met de eigenaar, verwerk feedback op visuele identiteit, content en gebruikservaring en werk de homepage responsive en inhoudelijk correct uit. Pas na goedkeuring van de visuele frontend start ik met de technische beheeromgeving en backend.</t>
-  </si>
-  <si>
-    <t>In Sprint 2 leverde ik het eerste werkende prototype van mijn vernieuwde portfoliowebsite op en presenteerde ik dit, samen met de gebruikte AI-systemen, aan Ronald Boiten. Ik liet zien hoe zijn grafische stijl en kleurgebruik in het ontwerp waren verwerkt en welke AI-tools ik daarvoor had ingezet. Ronald gaf concrete feedback op de fotografie, de teksten en de typografie, die ik direct heb vertaald naar aanpassingen voor Sprint 3. Daarmee heb ik niet alleen een praktijkgerichte AI-oplossing gerealiseerd, maar deze ook daadwerkelijk gepresenteerd aan een echte opdrachtgever en verwerkt in een concreet vervolgplan.</t>
-  </si>
-  <si>
-    <t>Ook in Sprint 2 koos ik per taak een andere tool. Voor de Learning Story rondom AI-agents volgde ik de DataCamp-cursus "Introduction to AI Agents" en vergeleek ik een agentic aanpak met mijn huidige werkwijze. Voor het onderzoek naar Blue Current combineerde ik deskresearch met een LLM om gerichte AI-kansen te formuleren voor het intakegesprek. Voor het prototype van de portfoliowebsite gebruikte ik opnieuw Visual Studio Code, GitHub en Vercel om de website live te zetten, en liet ik het resultaat beoordelen door Ronald Boiten. Zo zette ik per onderdeel bewust de tool in die het beste bij de taak paste.</t>
-  </si>
-  <si>
-    <t>Ik stuurde Sprint 2 grotendeels zelf aan. Ik koos zelf de DataCamp-cursus om mijn kennis over AI-agents te verdiepen, plande zelf het onderzoek naar Blue Current en de bijbehorende vragenlijst, en regelde zelfstandig de afspraak met Ronald Boiten om het prototype te bespreken. Na de feedback van Shahmeer en Ronald bepaalde ik zelf mijn vervolgstappen: eerst gebruikersvalidatie van het ontwerp, daarna pas de technische beheeromgeving. Ik hield dus zelf overzicht over mijn planning en stuurde bij op basis van de feedback die ik kreeg, zonder dat iemand mij een vast stappenplan gaf.</t>
-  </si>
-  <si>
-    <t>SPRINT 3</t>
-  </si>
-  <si>
     <t>SPRINT 4</t>
   </si>
   <si>
@@ -363,26 +415,17 @@
   </si>
   <si>
     <t>O</t>
-  </si>
-  <si>
-    <t>1. Een compact onderzoeksverslag met daarin de kernactiviteiten en propositie van Blue Current, en de huidige technologie- en laadinfrastructuurcontext.
-2. Minimaal 3 concrete AI-kansen/use cases uitgewerkt (bijv. slim laden/netcongestie, voorspellend onderhoud, geautomatiseerde support).
-3. Een gestructureerde vragenlijst (5–8 vragen) voor het intakegesprek met Blue Current.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. DataCamp-cursus "Introduction to AI Agents" succesvol afgerond, inclusief certificaat/bewijs van afronding in logboek.
-2. Een geschreven samenvatting waar de stof besproken wordt en je ten alle tijden de stof terug kan vinden
-3. De samenvatting is toegevoegd aan mijn portfolio om deze altijd bij de hand te hebben. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="166" formatCode="dd\-mm\-yy"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -419,14 +462,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="0" tint="-0.34998626667073579"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -521,7 +556,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -977,12 +1012,56 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF888888"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF888888"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF888888"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF888888"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF888888"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF888888"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF888888"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF888888"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1021,224 +1100,244 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="7" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="7" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="7" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1574,8 +1673,8 @@
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{00000000-000C-0000-FFFF-FFFF19000000}" name="Tabel7" displayName="Tabel7" ref="A25:D27" totalsRowShown="0">
-  <autoFilter ref="A25:D27" xr:uid="{00000000-0009-0000-0100-00001A000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{00000000-000C-0000-FFFF-FFFF19000000}" name="Tabel7" displayName="Tabel7" ref="A25:D28" totalsRowShown="0">
+  <autoFilter ref="A25:D28" xr:uid="{00000000-0009-0000-0100-00001A000000}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -2251,18 +2350,18 @@
       <c r="A9" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="102" t="s">
+      <c r="B9" s="107" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="103"/>
-      <c r="D9" s="103"/>
-      <c r="E9" s="103"/>
-      <c r="F9" s="103"/>
-      <c r="G9" s="103"/>
-      <c r="H9" s="103"/>
-      <c r="I9" s="103"/>
-      <c r="J9" s="103"/>
-      <c r="K9" s="103"/>
+      <c r="C9" s="108"/>
+      <c r="D9" s="108"/>
+      <c r="E9" s="108"/>
+      <c r="F9" s="108"/>
+      <c r="G9" s="108"/>
+      <c r="H9" s="108"/>
+      <c r="I9" s="108"/>
+      <c r="J9" s="108"/>
+      <c r="K9" s="109"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2277,7 +2376,7 @@
     <hyperlink ref="I1" location="Logboek!A141" display="Sprint 6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="J1" location="Logboek!A169" display="Sprint 7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="K1" location="Logboek!A197" display="Sprint 8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B9" r:id="rId1" xr:uid="{ACFFE906-FD52-644C-B2F0-667A25B82A49}"/>
+    <hyperlink ref="B9" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2296,12 +2395,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="110" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
-      <c r="D1" s="106"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="112"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A2" s="16"/>
@@ -2553,319 +2652,359 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="31"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="50"/>
-      <c r="D26" s="50"/>
-    </row>
-    <row r="27" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="51"/>
-      <c r="B27" s="52"/>
-      <c r="C27" s="50"/>
-      <c r="D27" s="50"/>
-    </row>
-    <row r="28" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="37"/>
-      <c r="B28" s="37"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
+    <row r="26" spans="1:4" ht="87" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="101">
+        <v>46281</v>
+      </c>
+      <c r="B26" s="102" t="s">
+        <v>67</v>
+      </c>
+      <c r="C26" s="50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" s="50" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="60" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="101">
+        <v>46281</v>
+      </c>
+      <c r="B27" s="102" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="D27" s="50" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="101">
+        <v>46281</v>
+      </c>
+      <c r="B28" s="102" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" s="50" t="s">
+        <v>74</v>
+      </c>
+      <c r="D28" s="50" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="104" t="s">
-        <v>67</v>
-      </c>
-      <c r="B29" s="104"/>
-      <c r="C29" s="104"/>
-      <c r="D29" s="104"/>
+      <c r="A29" s="113" t="s">
+        <v>76</v>
+      </c>
+      <c r="B29" s="114"/>
+      <c r="C29" s="114"/>
+      <c r="D29" s="115"/>
     </row>
     <row r="30" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="53"/>
-      <c r="B30" s="53"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="53"/>
+      <c r="A30" s="52"/>
+      <c r="B30" s="52"/>
+      <c r="C30" s="52"/>
+      <c r="D30" s="52"/>
     </row>
     <row r="31" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="B31" s="54"/>
-      <c r="C31" s="54"/>
+      <c r="A31" s="53" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" s="53"/>
+      <c r="C31" s="53"/>
       <c r="D31" s="18" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="55" t="s">
+      <c r="A32" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="B32" s="56" t="s">
+      <c r="B32" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="C32" s="56" t="s">
+      <c r="C32" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="D32" s="57" t="s">
+      <c r="D32" s="56" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="141" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="58" t="s">
+      <c r="A33" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="59" t="s">
-        <v>69</v>
-      </c>
-      <c r="C33" s="60" t="s">
+      <c r="B33" s="58" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="59" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33" s="60" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="143" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="57" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34" s="58" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" s="59" t="s">
+        <v>82</v>
+      </c>
+      <c r="D34" s="60" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="125" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="57" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="C35" s="59" t="s">
+        <v>85</v>
+      </c>
+      <c r="D35" s="60" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="57"/>
+      <c r="B36" s="58"/>
+      <c r="C36" s="59"/>
+      <c r="D36" s="60"/>
+    </row>
+    <row r="37" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="61"/>
+      <c r="B37" s="62"/>
+      <c r="C37" s="63"/>
+      <c r="D37" s="64"/>
+    </row>
+    <row r="38" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="52"/>
+      <c r="B38" s="52"/>
+      <c r="C38" s="52"/>
+      <c r="D38" s="52"/>
+    </row>
+    <row r="39" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="53" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" s="53"/>
+      <c r="C39" s="53"/>
+      <c r="D39" s="53"/>
+    </row>
+    <row r="40" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="54" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40" s="55" t="s">
+        <v>41</v>
+      </c>
+      <c r="D40" s="56" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="65">
+        <v>46288</v>
+      </c>
+      <c r="B41" s="59" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41" s="60" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="82.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="66">
+        <v>46292</v>
+      </c>
+      <c r="B42" s="67" t="s">
+        <v>90</v>
+      </c>
+      <c r="C42" s="67" t="s">
+        <v>91</v>
+      </c>
+      <c r="D42" s="68" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="69"/>
+      <c r="B43" s="70"/>
+      <c r="C43" s="70"/>
+      <c r="D43" s="71"/>
+    </row>
+    <row r="44" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="72" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" s="72"/>
+      <c r="C44" s="72"/>
+      <c r="D44" s="72"/>
+    </row>
+    <row r="45" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="54" t="s">
+        <v>0</v>
+      </c>
+      <c r="B45" s="55" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" s="55" t="s">
+        <v>45</v>
+      </c>
+      <c r="D45" s="56" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="73" t="s">
+        <v>47</v>
+      </c>
+      <c r="B46" s="74" t="s">
+        <v>48</v>
+      </c>
+      <c r="C46" s="75" t="s">
+        <v>56</v>
+      </c>
+      <c r="D46" s="60"/>
+    </row>
+    <row r="47" spans="1:4" ht="170" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="73" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="74" t="s">
+        <v>52</v>
+      </c>
+      <c r="C47" s="75" t="s">
+        <v>49</v>
+      </c>
+      <c r="D47" s="60" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="73" t="s">
+        <v>54</v>
+      </c>
+      <c r="B48" s="74" t="s">
+        <v>55</v>
+      </c>
+      <c r="C48" s="75" t="s">
+        <v>56</v>
+      </c>
+      <c r="D48" s="60"/>
+    </row>
+    <row r="49" spans="1:4" ht="169" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="73" t="s">
+        <v>57</v>
+      </c>
+      <c r="B49" s="74" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" s="75" t="s">
+        <v>49</v>
+      </c>
+      <c r="D49" s="60" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="175" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="76" t="s">
+        <v>60</v>
+      </c>
+      <c r="B50" s="77" t="s">
+        <v>61</v>
+      </c>
+      <c r="C50" s="78" t="s">
+        <v>49</v>
+      </c>
+      <c r="D50" s="64" t="s">
         <v>95</v>
       </c>
-      <c r="D33" s="61" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="143" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="58" t="s">
-        <v>26</v>
-      </c>
-      <c r="B34" s="59" t="s">
-        <v>71</v>
-      </c>
-      <c r="C34" s="60" t="s">
-        <v>94</v>
-      </c>
-      <c r="D34" s="61" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="125" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="58" t="s">
-        <v>30</v>
-      </c>
-      <c r="B35" s="59" t="s">
-        <v>73</v>
-      </c>
-      <c r="C35" s="60" t="s">
-        <v>74</v>
-      </c>
-      <c r="D35" s="61" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="58"/>
-      <c r="B36" s="59"/>
-      <c r="C36" s="60"/>
-      <c r="D36" s="61"/>
-    </row>
-    <row r="37" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="62"/>
-      <c r="B37" s="63"/>
-      <c r="C37" s="64"/>
-      <c r="D37" s="65"/>
-    </row>
-    <row r="38" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="53"/>
-      <c r="B38" s="53"/>
-      <c r="C38" s="53"/>
-      <c r="D38" s="53"/>
-    </row>
-    <row r="39" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="54" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39" s="54"/>
-      <c r="C39" s="54"/>
-      <c r="D39" s="54"/>
-    </row>
-    <row r="40" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="55" t="s">
+    </row>
+    <row r="51" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="52"/>
+      <c r="B51" s="79"/>
+      <c r="C51" s="80"/>
+      <c r="D51" s="80"/>
+    </row>
+    <row r="52" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="B52" s="81"/>
+      <c r="C52" s="82"/>
+      <c r="D52" s="82"/>
+    </row>
+    <row r="53" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="56" t="s">
-        <v>40</v>
-      </c>
-      <c r="C40" s="56" t="s">
-        <v>41</v>
-      </c>
-      <c r="D40" s="57" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="66">
-        <v>46288</v>
-      </c>
-      <c r="B41" s="60" t="s">
-        <v>78</v>
-      </c>
-      <c r="C41" s="60" t="s">
-        <v>79</v>
-      </c>
-      <c r="D41" s="61" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="82.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="67">
-        <v>46292</v>
-      </c>
-      <c r="B42" s="68" t="s">
-        <v>81</v>
-      </c>
-      <c r="C42" s="68" t="s">
-        <v>82</v>
-      </c>
-      <c r="D42" s="69" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="70"/>
-      <c r="B43" s="71"/>
-      <c r="C43" s="71"/>
-      <c r="D43" s="72"/>
-    </row>
-    <row r="44" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="73" t="s">
-        <v>43</v>
-      </c>
-      <c r="B44" s="73"/>
-      <c r="C44" s="73"/>
-      <c r="D44" s="73"/>
-    </row>
-    <row r="45" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B45" s="56" t="s">
-        <v>44</v>
-      </c>
-      <c r="C45" s="56" t="s">
-        <v>45</v>
-      </c>
-      <c r="D45" s="57" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="74" t="s">
-        <v>47</v>
-      </c>
-      <c r="B46" s="75" t="s">
-        <v>48</v>
-      </c>
-      <c r="C46" s="76" t="s">
-        <v>56</v>
-      </c>
-      <c r="D46" s="61"/>
-    </row>
-    <row r="47" spans="1:4" ht="170" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="74" t="s">
-        <v>51</v>
-      </c>
-      <c r="B47" s="75" t="s">
-        <v>52</v>
-      </c>
-      <c r="C47" s="76" t="s">
-        <v>49</v>
-      </c>
-      <c r="D47" s="61" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="74" t="s">
-        <v>54</v>
-      </c>
-      <c r="B48" s="75" t="s">
-        <v>55</v>
-      </c>
-      <c r="C48" s="76" t="s">
-        <v>56</v>
-      </c>
-      <c r="D48" s="61"/>
-    </row>
-    <row r="49" spans="1:4" ht="169" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="74" t="s">
-        <v>57</v>
-      </c>
-      <c r="B49" s="75" t="s">
-        <v>58</v>
-      </c>
-      <c r="C49" s="76" t="s">
-        <v>49</v>
-      </c>
-      <c r="D49" s="61" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="175" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="77" t="s">
-        <v>60</v>
-      </c>
-      <c r="B50" s="78" t="s">
-        <v>61</v>
-      </c>
-      <c r="C50" s="79" t="s">
-        <v>49</v>
-      </c>
-      <c r="D50" s="65" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="53"/>
-      <c r="B51" s="80"/>
-      <c r="C51" s="81"/>
-      <c r="D51" s="81"/>
-    </row>
-    <row r="52" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="54" t="s">
-        <v>63</v>
-      </c>
-      <c r="B52" s="82"/>
-      <c r="C52" s="83"/>
-      <c r="D52" s="83"/>
-    </row>
-    <row r="53" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="55" t="s">
-        <v>39</v>
-      </c>
-      <c r="B53" s="84" t="s">
+      <c r="B53" s="83" t="s">
         <v>64</v>
       </c>
-      <c r="C53" s="85" t="s">
+      <c r="C53" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="D53" s="57" t="s">
+      <c r="D53" s="56" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="66"/>
-      <c r="B54" s="60"/>
-      <c r="C54" s="60"/>
-      <c r="D54" s="61"/>
-    </row>
-    <row r="55" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="86"/>
-      <c r="B55" s="87"/>
-      <c r="C55" s="68"/>
-      <c r="D55" s="69"/>
+    <row r="54" spans="1:4" ht="60" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="103">
+        <v>46294</v>
+      </c>
+      <c r="B54" s="104" t="s">
+        <v>96</v>
+      </c>
+      <c r="C54" s="105" t="s">
+        <v>97</v>
+      </c>
+      <c r="D54" s="106" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="73.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="103">
+        <v>46294</v>
+      </c>
+      <c r="B55" s="104" t="s">
+        <v>99</v>
+      </c>
+      <c r="C55" s="105" t="s">
+        <v>100</v>
+      </c>
+      <c r="D55" s="106" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="56" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="70"/>
-      <c r="B56" s="71"/>
-      <c r="C56" s="71"/>
-      <c r="D56" s="72"/>
+      <c r="A56" s="69"/>
+      <c r="B56" s="70"/>
+      <c r="C56" s="70"/>
+      <c r="D56" s="71"/>
     </row>
     <row r="57" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="105" t="s">
-        <v>87</v>
-      </c>
-      <c r="B57" s="105"/>
-      <c r="C57" s="105"/>
-      <c r="D57" s="105"/>
+      <c r="A57" s="116" t="s">
+        <v>102</v>
+      </c>
+      <c r="B57" s="114"/>
+      <c r="C57" s="114"/>
+      <c r="D57" s="115"/>
     </row>
     <row r="58" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A58" s="16"/>
@@ -2875,7 +3014,7 @@
     </row>
     <row r="59" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A59" s="17" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="B59" s="17"/>
       <c r="C59" s="17"/>
@@ -2902,61 +3041,61 @@
         <v>30</v>
       </c>
       <c r="B61" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C61" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D61" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A62" s="22"/>
       <c r="B62" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C62" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D62" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A63" s="22"/>
       <c r="B63" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C63" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D63" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A64" s="22"/>
       <c r="B64" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C64" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D64" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A65" s="26"/>
       <c r="B65" s="27" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C65" s="28" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D65" s="29" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
@@ -2995,15 +3134,15 @@
     </row>
     <row r="70" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A70" s="35"/>
-      <c r="B70" s="88"/>
-      <c r="C70" s="88"/>
-      <c r="D70" s="89"/>
+      <c r="B70" s="87"/>
+      <c r="C70" s="87"/>
+      <c r="D70" s="88"/>
     </row>
     <row r="71" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="90"/>
+      <c r="A71" s="89"/>
       <c r="B71" s="37"/>
       <c r="C71" s="37"/>
-      <c r="D71" s="91"/>
+      <c r="D71" s="90"/>
     </row>
     <row r="72" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A72" s="38" t="s">
@@ -3123,297 +3262,297 @@
     </row>
     <row r="83" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A83" s="51"/>
-      <c r="B83" s="92"/>
+      <c r="B83" s="91"/>
       <c r="C83" s="50"/>
       <c r="D83" s="50"/>
     </row>
     <row r="84" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="90"/>
+      <c r="A84" s="89"/>
       <c r="B84" s="37"/>
       <c r="C84" s="37"/>
-      <c r="D84" s="91"/>
+      <c r="D84" s="90"/>
     </row>
     <row r="85" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="104" t="s">
-        <v>88</v>
-      </c>
-      <c r="B85" s="104"/>
-      <c r="C85" s="104"/>
-      <c r="D85" s="104"/>
+      <c r="A85" s="113" t="s">
+        <v>105</v>
+      </c>
+      <c r="B85" s="114"/>
+      <c r="C85" s="114"/>
+      <c r="D85" s="115"/>
     </row>
     <row r="86" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="53"/>
-      <c r="B86" s="53"/>
-      <c r="C86" s="53"/>
-      <c r="D86" s="53"/>
+      <c r="A86" s="52"/>
+      <c r="B86" s="52"/>
+      <c r="C86" s="52"/>
+      <c r="D86" s="52"/>
     </row>
     <row r="87" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="B87" s="54"/>
-      <c r="C87" s="54"/>
+      <c r="A87" s="53" t="s">
+        <v>77</v>
+      </c>
+      <c r="B87" s="53"/>
+      <c r="C87" s="53"/>
       <c r="D87" s="18" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="55" t="s">
+      <c r="A88" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="B88" s="56" t="s">
+      <c r="B88" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="C88" s="56" t="s">
+      <c r="C88" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="D88" s="57" t="s">
+      <c r="D88" s="56" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="58" t="s">
+      <c r="A89" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="B89" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C89" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D89" s="61" t="s">
-        <v>77</v>
+      <c r="B89" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C89" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D89" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="58"/>
-      <c r="B90" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C90" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D90" s="61" t="s">
-        <v>77</v>
+      <c r="A90" s="57"/>
+      <c r="B90" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C90" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D90" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="58"/>
-      <c r="B91" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C91" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D91" s="61" t="s">
-        <v>77</v>
+      <c r="A91" s="57"/>
+      <c r="B91" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C91" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D91" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="58"/>
-      <c r="B92" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C92" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D92" s="61" t="s">
-        <v>77</v>
+      <c r="A92" s="57"/>
+      <c r="B92" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C92" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D92" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="62"/>
-      <c r="B93" s="63" t="s">
-        <v>76</v>
-      </c>
-      <c r="C93" s="64" t="s">
-        <v>77</v>
-      </c>
-      <c r="D93" s="65" t="s">
-        <v>77</v>
+      <c r="A93" s="61"/>
+      <c r="B93" s="62" t="s">
+        <v>103</v>
+      </c>
+      <c r="C93" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="D93" s="64" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="53"/>
-      <c r="B94" s="53"/>
-      <c r="C94" s="53"/>
-      <c r="D94" s="53"/>
+      <c r="A94" s="52"/>
+      <c r="B94" s="52"/>
+      <c r="C94" s="52"/>
+      <c r="D94" s="52"/>
     </row>
     <row r="95" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="54" t="s">
+      <c r="A95" s="53" t="s">
         <v>38</v>
       </c>
-      <c r="B95" s="54"/>
-      <c r="C95" s="54"/>
-      <c r="D95" s="54"/>
+      <c r="B95" s="53"/>
+      <c r="C95" s="53"/>
+      <c r="D95" s="53"/>
     </row>
     <row r="96" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="55" t="s">
+      <c r="A96" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="B96" s="56" t="s">
+      <c r="B96" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="C96" s="56" t="s">
+      <c r="C96" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="D96" s="57" t="s">
+      <c r="D96" s="56" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="66"/>
-      <c r="B97" s="60"/>
-      <c r="C97" s="60"/>
-      <c r="D97" s="61"/>
+      <c r="A97" s="65"/>
+      <c r="B97" s="59"/>
+      <c r="C97" s="59"/>
+      <c r="D97" s="60"/>
     </row>
     <row r="98" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="67"/>
-      <c r="B98" s="68"/>
-      <c r="C98" s="68"/>
-      <c r="D98" s="69"/>
+      <c r="A98" s="66"/>
+      <c r="B98" s="67"/>
+      <c r="C98" s="67"/>
+      <c r="D98" s="68"/>
     </row>
     <row r="99" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="70"/>
-      <c r="B99" s="71"/>
-      <c r="C99" s="71"/>
-      <c r="D99" s="72"/>
+      <c r="A99" s="69"/>
+      <c r="B99" s="70"/>
+      <c r="C99" s="70"/>
+      <c r="D99" s="71"/>
     </row>
     <row r="100" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="73" t="s">
+      <c r="A100" s="72" t="s">
         <v>43</v>
       </c>
-      <c r="B100" s="73"/>
-      <c r="C100" s="73"/>
-      <c r="D100" s="73"/>
+      <c r="B100" s="72"/>
+      <c r="C100" s="72"/>
+      <c r="D100" s="72"/>
     </row>
     <row r="101" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="55" t="s">
+      <c r="A101" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B101" s="56" t="s">
+      <c r="B101" s="55" t="s">
         <v>44</v>
       </c>
-      <c r="C101" s="56" t="s">
+      <c r="C101" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="D101" s="57" t="s">
+      <c r="D101" s="56" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="102" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="74" t="s">
+      <c r="A102" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="B102" s="75" t="s">
+      <c r="B102" s="74" t="s">
         <v>48</v>
       </c>
-      <c r="C102" s="76" t="s">
+      <c r="C102" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D102" s="61"/>
+      <c r="D102" s="60"/>
     </row>
     <row r="103" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A103" s="74" t="s">
+      <c r="A103" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="B103" s="75" t="s">
+      <c r="B103" s="74" t="s">
         <v>52</v>
       </c>
-      <c r="C103" s="76" t="s">
+      <c r="C103" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D103" s="61"/>
+      <c r="D103" s="60"/>
     </row>
     <row r="104" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A104" s="74" t="s">
+      <c r="A104" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="B104" s="75" t="s">
+      <c r="B104" s="74" t="s">
         <v>55</v>
       </c>
-      <c r="C104" s="76" t="s">
+      <c r="C104" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D104" s="61"/>
+      <c r="D104" s="60"/>
     </row>
     <row r="105" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A105" s="74" t="s">
+      <c r="A105" s="73" t="s">
         <v>57</v>
       </c>
-      <c r="B105" s="75" t="s">
+      <c r="B105" s="74" t="s">
         <v>58</v>
       </c>
-      <c r="C105" s="76" t="s">
+      <c r="C105" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D105" s="61"/>
+      <c r="D105" s="60"/>
     </row>
     <row r="106" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A106" s="77" t="s">
+      <c r="A106" s="76" t="s">
         <v>60</v>
       </c>
-      <c r="B106" s="78" t="s">
+      <c r="B106" s="77" t="s">
         <v>61</v>
       </c>
-      <c r="C106" s="79" t="s">
+      <c r="C106" s="78" t="s">
         <v>56</v>
       </c>
-      <c r="D106" s="65"/>
+      <c r="D106" s="64"/>
     </row>
     <row r="107" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="53"/>
-      <c r="B107" s="80"/>
-      <c r="C107" s="81"/>
-      <c r="D107" s="81"/>
+      <c r="A107" s="52"/>
+      <c r="B107" s="79"/>
+      <c r="C107" s="80"/>
+      <c r="D107" s="80"/>
     </row>
     <row r="108" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A108" s="54" t="s">
+      <c r="A108" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="B108" s="82"/>
-      <c r="C108" s="83"/>
-      <c r="D108" s="83"/>
+      <c r="B108" s="81"/>
+      <c r="C108" s="82"/>
+      <c r="D108" s="82"/>
     </row>
     <row r="109" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="55" t="s">
+      <c r="A109" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="B109" s="84" t="s">
+      <c r="B109" s="83" t="s">
         <v>64</v>
       </c>
-      <c r="C109" s="85" t="s">
+      <c r="C109" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="D109" s="57" t="s">
+      <c r="D109" s="56" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="110" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="66"/>
-      <c r="B110" s="60"/>
-      <c r="C110" s="60"/>
-      <c r="D110" s="61"/>
+      <c r="A110" s="65"/>
+      <c r="B110" s="59"/>
+      <c r="C110" s="59"/>
+      <c r="D110" s="60"/>
     </row>
     <row r="111" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A111" s="86"/>
-      <c r="B111" s="87"/>
-      <c r="C111" s="68"/>
-      <c r="D111" s="69"/>
+      <c r="A111" s="85"/>
+      <c r="B111" s="86"/>
+      <c r="C111" s="67"/>
+      <c r="D111" s="68"/>
     </row>
     <row r="112" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" s="70"/>
-      <c r="B112" s="71"/>
-      <c r="C112" s="71"/>
-      <c r="D112" s="72"/>
+      <c r="A112" s="69"/>
+      <c r="B112" s="70"/>
+      <c r="C112" s="70"/>
+      <c r="D112" s="71"/>
     </row>
     <row r="113" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A113" s="105" t="s">
-        <v>89</v>
-      </c>
-      <c r="B113" s="105"/>
-      <c r="C113" s="105"/>
-      <c r="D113" s="105"/>
+      <c r="A113" s="116" t="s">
+        <v>106</v>
+      </c>
+      <c r="B113" s="114"/>
+      <c r="C113" s="114"/>
+      <c r="D113" s="115"/>
     </row>
     <row r="114" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A114" s="16"/>
@@ -3423,7 +3562,7 @@
     </row>
     <row r="115" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A115" s="17" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="B115" s="17"/>
       <c r="C115" s="17"/>
@@ -3450,61 +3589,61 @@
         <v>30</v>
       </c>
       <c r="B117" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C117" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D117" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A118" s="22"/>
       <c r="B118" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C118" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D118" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="119" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A119" s="22"/>
       <c r="B119" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C119" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D119" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A120" s="22"/>
       <c r="B120" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C120" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D120" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="121" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A121" s="26"/>
       <c r="B121" s="27" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C121" s="28" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D121" s="29" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="122" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
@@ -3543,15 +3682,15 @@
     </row>
     <row r="126" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A126" s="35"/>
-      <c r="B126" s="88"/>
-      <c r="C126" s="88"/>
-      <c r="D126" s="89"/>
+      <c r="B126" s="87"/>
+      <c r="C126" s="87"/>
+      <c r="D126" s="88"/>
     </row>
     <row r="127" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="90"/>
+      <c r="A127" s="89"/>
       <c r="B127" s="37"/>
       <c r="C127" s="37"/>
-      <c r="D127" s="91"/>
+      <c r="D127" s="90"/>
     </row>
     <row r="128" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A128" s="38" t="s">
@@ -3671,297 +3810,297 @@
     </row>
     <row r="139" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A139" s="51"/>
-      <c r="B139" s="92"/>
+      <c r="B139" s="91"/>
       <c r="C139" s="50"/>
       <c r="D139" s="50"/>
     </row>
     <row r="140" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="90"/>
+      <c r="A140" s="89"/>
       <c r="B140" s="37"/>
       <c r="C140" s="37"/>
-      <c r="D140" s="91"/>
+      <c r="D140" s="90"/>
     </row>
     <row r="141" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="104" t="s">
-        <v>90</v>
-      </c>
-      <c r="B141" s="104"/>
-      <c r="C141" s="104"/>
-      <c r="D141" s="104"/>
+      <c r="A141" s="113" t="s">
+        <v>107</v>
+      </c>
+      <c r="B141" s="114"/>
+      <c r="C141" s="114"/>
+      <c r="D141" s="115"/>
     </row>
     <row r="142" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A142" s="53"/>
-      <c r="B142" s="53"/>
-      <c r="C142" s="53"/>
-      <c r="D142" s="53"/>
+      <c r="A142" s="52"/>
+      <c r="B142" s="52"/>
+      <c r="C142" s="52"/>
+      <c r="D142" s="52"/>
     </row>
     <row r="143" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A143" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="B143" s="54"/>
-      <c r="C143" s="54"/>
+      <c r="A143" s="53" t="s">
+        <v>77</v>
+      </c>
+      <c r="B143" s="53"/>
+      <c r="C143" s="53"/>
       <c r="D143" s="18" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="144" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="55" t="s">
+      <c r="A144" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="B144" s="56" t="s">
+      <c r="B144" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="C144" s="56" t="s">
+      <c r="C144" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="D144" s="57" t="s">
+      <c r="D144" s="56" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="145" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="58" t="s">
+      <c r="A145" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="B145" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C145" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D145" s="61" t="s">
-        <v>77</v>
+      <c r="B145" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C145" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D145" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="146" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="58"/>
-      <c r="B146" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C146" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D146" s="61" t="s">
-        <v>77</v>
+      <c r="A146" s="57"/>
+      <c r="B146" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C146" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D146" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="58"/>
-      <c r="B147" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C147" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D147" s="61" t="s">
-        <v>77</v>
+      <c r="A147" s="57"/>
+      <c r="B147" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C147" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D147" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="148" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="58"/>
-      <c r="B148" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C148" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D148" s="61" t="s">
-        <v>77</v>
+      <c r="A148" s="57"/>
+      <c r="B148" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C148" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D148" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="149" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="62"/>
-      <c r="B149" s="63" t="s">
-        <v>76</v>
-      </c>
-      <c r="C149" s="64" t="s">
-        <v>77</v>
-      </c>
-      <c r="D149" s="65" t="s">
-        <v>77</v>
+      <c r="A149" s="61"/>
+      <c r="B149" s="62" t="s">
+        <v>103</v>
+      </c>
+      <c r="C149" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="D149" s="64" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="150" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A150" s="53"/>
-      <c r="B150" s="53"/>
-      <c r="C150" s="53"/>
-      <c r="D150" s="53"/>
+      <c r="A150" s="52"/>
+      <c r="B150" s="52"/>
+      <c r="C150" s="52"/>
+      <c r="D150" s="52"/>
     </row>
     <row r="151" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="54" t="s">
+      <c r="A151" s="53" t="s">
         <v>38</v>
       </c>
-      <c r="B151" s="54"/>
-      <c r="C151" s="54"/>
-      <c r="D151" s="54"/>
+      <c r="B151" s="53"/>
+      <c r="C151" s="53"/>
+      <c r="D151" s="53"/>
     </row>
     <row r="152" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="55" t="s">
+      <c r="A152" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="B152" s="56" t="s">
+      <c r="B152" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="C152" s="56" t="s">
+      <c r="C152" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="D152" s="57" t="s">
+      <c r="D152" s="56" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="153" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="66"/>
-      <c r="B153" s="60"/>
-      <c r="C153" s="60"/>
-      <c r="D153" s="61"/>
+      <c r="A153" s="65"/>
+      <c r="B153" s="59"/>
+      <c r="C153" s="59"/>
+      <c r="D153" s="60"/>
     </row>
     <row r="154" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="67"/>
-      <c r="B154" s="68"/>
-      <c r="C154" s="68"/>
-      <c r="D154" s="69"/>
+      <c r="A154" s="66"/>
+      <c r="B154" s="67"/>
+      <c r="C154" s="67"/>
+      <c r="D154" s="68"/>
     </row>
     <row r="155" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="70"/>
-      <c r="B155" s="71"/>
-      <c r="C155" s="71"/>
-      <c r="D155" s="72"/>
+      <c r="A155" s="69"/>
+      <c r="B155" s="70"/>
+      <c r="C155" s="70"/>
+      <c r="D155" s="71"/>
     </row>
     <row r="156" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="93" t="s">
+      <c r="A156" s="92" t="s">
         <v>43</v>
       </c>
-      <c r="B156" s="94"/>
-      <c r="C156" s="94"/>
-      <c r="D156" s="95"/>
+      <c r="B156" s="93"/>
+      <c r="C156" s="93"/>
+      <c r="D156" s="94"/>
     </row>
     <row r="157" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A157" s="96" t="s">
+      <c r="A157" s="95" t="s">
         <v>0</v>
       </c>
-      <c r="B157" s="97" t="s">
+      <c r="B157" s="96" t="s">
         <v>44</v>
       </c>
-      <c r="C157" s="97" t="s">
+      <c r="C157" s="96" t="s">
         <v>45</v>
       </c>
-      <c r="D157" s="98" t="s">
+      <c r="D157" s="97" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="158" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="74" t="s">
+      <c r="A158" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="B158" s="75" t="s">
+      <c r="B158" s="74" t="s">
         <v>48</v>
       </c>
-      <c r="C158" s="76" t="s">
+      <c r="C158" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D158" s="61"/>
+      <c r="D158" s="60"/>
     </row>
     <row r="159" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="74" t="s">
+      <c r="A159" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="B159" s="75" t="s">
+      <c r="B159" s="74" t="s">
         <v>52</v>
       </c>
-      <c r="C159" s="76" t="s">
+      <c r="C159" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D159" s="61"/>
+      <c r="D159" s="60"/>
     </row>
     <row r="160" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="74" t="s">
+      <c r="A160" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="B160" s="75" t="s">
+      <c r="B160" s="74" t="s">
         <v>55</v>
       </c>
-      <c r="C160" s="76" t="s">
+      <c r="C160" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D160" s="61"/>
+      <c r="D160" s="60"/>
     </row>
     <row r="161" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A161" s="74" t="s">
+      <c r="A161" s="73" t="s">
         <v>57</v>
       </c>
-      <c r="B161" s="75" t="s">
+      <c r="B161" s="74" t="s">
         <v>58</v>
       </c>
-      <c r="C161" s="76" t="s">
+      <c r="C161" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D161" s="61"/>
+      <c r="D161" s="60"/>
     </row>
     <row r="162" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A162" s="77" t="s">
+      <c r="A162" s="76" t="s">
         <v>60</v>
       </c>
-      <c r="B162" s="78" t="s">
+      <c r="B162" s="77" t="s">
         <v>61</v>
       </c>
-      <c r="C162" s="79" t="s">
+      <c r="C162" s="78" t="s">
         <v>56</v>
       </c>
-      <c r="D162" s="65"/>
+      <c r="D162" s="64"/>
     </row>
     <row r="163" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="53"/>
-      <c r="B163" s="80"/>
-      <c r="C163" s="81"/>
-      <c r="D163" s="81"/>
+      <c r="A163" s="52"/>
+      <c r="B163" s="79"/>
+      <c r="C163" s="80"/>
+      <c r="D163" s="80"/>
     </row>
     <row r="164" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="54" t="s">
+      <c r="A164" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="B164" s="82"/>
-      <c r="C164" s="83"/>
-      <c r="D164" s="83"/>
+      <c r="B164" s="81"/>
+      <c r="C164" s="82"/>
+      <c r="D164" s="82"/>
     </row>
     <row r="165" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A165" s="55" t="s">
+      <c r="A165" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="B165" s="84" t="s">
+      <c r="B165" s="83" t="s">
         <v>64</v>
       </c>
-      <c r="C165" s="85" t="s">
+      <c r="C165" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="D165" s="57" t="s">
+      <c r="D165" s="56" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="166" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A166" s="66"/>
-      <c r="B166" s="60"/>
-      <c r="C166" s="60"/>
-      <c r="D166" s="61"/>
+      <c r="A166" s="65"/>
+      <c r="B166" s="59"/>
+      <c r="C166" s="59"/>
+      <c r="D166" s="60"/>
     </row>
     <row r="167" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A167" s="86"/>
-      <c r="B167" s="87"/>
-      <c r="C167" s="68"/>
-      <c r="D167" s="69"/>
+      <c r="A167" s="85"/>
+      <c r="B167" s="86"/>
+      <c r="C167" s="67"/>
+      <c r="D167" s="68"/>
     </row>
     <row r="168" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A168" s="70"/>
-      <c r="B168" s="71"/>
-      <c r="C168" s="71"/>
-      <c r="D168" s="72"/>
+      <c r="A168" s="69"/>
+      <c r="B168" s="70"/>
+      <c r="C168" s="70"/>
+      <c r="D168" s="71"/>
     </row>
     <row r="169" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A169" s="105" t="s">
-        <v>91</v>
-      </c>
-      <c r="B169" s="105"/>
-      <c r="C169" s="105"/>
-      <c r="D169" s="105"/>
+      <c r="A169" s="116" t="s">
+        <v>108</v>
+      </c>
+      <c r="B169" s="114"/>
+      <c r="C169" s="114"/>
+      <c r="D169" s="115"/>
     </row>
     <row r="170" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A170" s="16"/>
@@ -3971,7 +4110,7 @@
     </row>
     <row r="171" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A171" s="17" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="B171" s="17"/>
       <c r="C171" s="17"/>
@@ -3998,61 +4137,61 @@
         <v>30</v>
       </c>
       <c r="B173" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C173" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D173" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="174" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A174" s="22"/>
       <c r="B174" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C174" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D174" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="175" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A175" s="22"/>
       <c r="B175" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C175" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D175" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="176" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A176" s="22"/>
       <c r="B176" s="25" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C176" s="23" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D176" s="24" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="177" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A177" s="26"/>
       <c r="B177" s="27" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C177" s="28" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D177" s="29" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="178" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
@@ -4091,15 +4230,15 @@
     </row>
     <row r="182" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A182" s="35"/>
-      <c r="B182" s="88"/>
-      <c r="C182" s="88"/>
-      <c r="D182" s="89"/>
+      <c r="B182" s="87"/>
+      <c r="C182" s="87"/>
+      <c r="D182" s="88"/>
     </row>
     <row r="183" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A183" s="90"/>
+      <c r="A183" s="89"/>
       <c r="B183" s="37"/>
       <c r="C183" s="37"/>
-      <c r="D183" s="91"/>
+      <c r="D183" s="90"/>
     </row>
     <row r="184" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A184" s="38" t="s">
@@ -4219,294 +4358,294 @@
     </row>
     <row r="195" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A195" s="51"/>
-      <c r="B195" s="92"/>
+      <c r="B195" s="91"/>
       <c r="C195" s="50"/>
       <c r="D195" s="50"/>
     </row>
     <row r="196" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A196" s="90"/>
+      <c r="A196" s="89"/>
       <c r="B196" s="37"/>
       <c r="C196" s="37"/>
-      <c r="D196" s="91"/>
+      <c r="D196" s="90"/>
     </row>
     <row r="197" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A197" s="104" t="s">
-        <v>92</v>
-      </c>
-      <c r="B197" s="104"/>
-      <c r="C197" s="104"/>
-      <c r="D197" s="104"/>
+      <c r="A197" s="113" t="s">
+        <v>109</v>
+      </c>
+      <c r="B197" s="114"/>
+      <c r="C197" s="114"/>
+      <c r="D197" s="115"/>
     </row>
     <row r="198" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A198" s="53"/>
-      <c r="B198" s="53"/>
-      <c r="C198" s="53"/>
-      <c r="D198" s="53"/>
+      <c r="A198" s="52"/>
+      <c r="B198" s="52"/>
+      <c r="C198" s="52"/>
+      <c r="D198" s="52"/>
     </row>
     <row r="199" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A199" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="B199" s="54"/>
-      <c r="C199" s="54"/>
+      <c r="A199" s="53" t="s">
+        <v>77</v>
+      </c>
+      <c r="B199" s="53"/>
+      <c r="C199" s="53"/>
       <c r="D199" s="18" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="200" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A200" s="55" t="s">
+      <c r="A200" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="B200" s="56" t="s">
+      <c r="B200" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="C200" s="56" t="s">
+      <c r="C200" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="D200" s="57" t="s">
+      <c r="D200" s="56" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="201" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A201" s="58" t="s">
+      <c r="A201" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="B201" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C201" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D201" s="61" t="s">
-        <v>77</v>
+      <c r="B201" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C201" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D201" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="202" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A202" s="58"/>
-      <c r="B202" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C202" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D202" s="61" t="s">
-        <v>77</v>
+      <c r="A202" s="57"/>
+      <c r="B202" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C202" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D202" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="203" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A203" s="58"/>
-      <c r="B203" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C203" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D203" s="61" t="s">
-        <v>77</v>
+      <c r="A203" s="57"/>
+      <c r="B203" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C203" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D203" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="204" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A204" s="58"/>
-      <c r="B204" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="C204" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="D204" s="61" t="s">
-        <v>77</v>
+      <c r="A204" s="57"/>
+      <c r="B204" s="58" t="s">
+        <v>103</v>
+      </c>
+      <c r="C204" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D204" s="60" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="205" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A205" s="62"/>
-      <c r="B205" s="63" t="s">
-        <v>76</v>
-      </c>
-      <c r="C205" s="64" t="s">
-        <v>77</v>
-      </c>
-      <c r="D205" s="65" t="s">
-        <v>77</v>
+      <c r="A205" s="61"/>
+      <c r="B205" s="62" t="s">
+        <v>103</v>
+      </c>
+      <c r="C205" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="D205" s="64" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="206" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A206" s="53"/>
-      <c r="B206" s="53"/>
-      <c r="C206" s="53"/>
-      <c r="D206" s="53"/>
+      <c r="A206" s="52"/>
+      <c r="B206" s="52"/>
+      <c r="C206" s="52"/>
+      <c r="D206" s="52"/>
     </row>
     <row r="207" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A207" s="54" t="s">
+      <c r="A207" s="53" t="s">
         <v>38</v>
       </c>
-      <c r="B207" s="54"/>
-      <c r="C207" s="54"/>
-      <c r="D207" s="54"/>
+      <c r="B207" s="53"/>
+      <c r="C207" s="53"/>
+      <c r="D207" s="53"/>
     </row>
     <row r="208" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A208" s="55" t="s">
+      <c r="A208" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="B208" s="56" t="s">
+      <c r="B208" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="C208" s="56" t="s">
+      <c r="C208" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="D208" s="57" t="s">
+      <c r="D208" s="56" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="209" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A209" s="66"/>
-      <c r="B209" s="60"/>
-      <c r="C209" s="60"/>
-      <c r="D209" s="61"/>
+      <c r="A209" s="65"/>
+      <c r="B209" s="59"/>
+      <c r="C209" s="59"/>
+      <c r="D209" s="60"/>
     </row>
     <row r="210" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A210" s="67"/>
-      <c r="B210" s="68"/>
-      <c r="C210" s="68"/>
-      <c r="D210" s="69"/>
+      <c r="A210" s="66"/>
+      <c r="B210" s="67"/>
+      <c r="C210" s="67"/>
+      <c r="D210" s="68"/>
     </row>
     <row r="211" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A211" s="70"/>
-      <c r="B211" s="71"/>
-      <c r="C211" s="71"/>
-      <c r="D211" s="72"/>
+      <c r="A211" s="69"/>
+      <c r="B211" s="70"/>
+      <c r="C211" s="70"/>
+      <c r="D211" s="71"/>
     </row>
     <row r="212" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A212" s="73" t="s">
+      <c r="A212" s="72" t="s">
         <v>43</v>
       </c>
-      <c r="B212" s="73"/>
-      <c r="C212" s="73"/>
-      <c r="D212" s="73"/>
+      <c r="B212" s="72"/>
+      <c r="C212" s="72"/>
+      <c r="D212" s="72"/>
     </row>
     <row r="213" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A213" s="55" t="s">
+      <c r="A213" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B213" s="56" t="s">
+      <c r="B213" s="55" t="s">
         <v>44</v>
       </c>
-      <c r="C213" s="56" t="s">
+      <c r="C213" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="D213" s="57" t="s">
+      <c r="D213" s="56" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="214" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A214" s="74" t="s">
+      <c r="A214" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="B214" s="75" t="s">
+      <c r="B214" s="74" t="s">
         <v>48</v>
       </c>
-      <c r="C214" s="76" t="s">
+      <c r="C214" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D214" s="61"/>
+      <c r="D214" s="60"/>
     </row>
     <row r="215" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A215" s="74" t="s">
+      <c r="A215" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="B215" s="75" t="s">
+      <c r="B215" s="74" t="s">
         <v>52</v>
       </c>
-      <c r="C215" s="76" t="s">
+      <c r="C215" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D215" s="61"/>
+      <c r="D215" s="60"/>
     </row>
     <row r="216" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A216" s="74" t="s">
+      <c r="A216" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="B216" s="75" t="s">
+      <c r="B216" s="74" t="s">
         <v>55</v>
       </c>
-      <c r="C216" s="76" t="s">
+      <c r="C216" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D216" s="61"/>
+      <c r="D216" s="60"/>
     </row>
     <row r="217" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A217" s="74" t="s">
+      <c r="A217" s="73" t="s">
         <v>57</v>
       </c>
-      <c r="B217" s="75" t="s">
+      <c r="B217" s="74" t="s">
         <v>58</v>
       </c>
-      <c r="C217" s="76" t="s">
+      <c r="C217" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="D217" s="61"/>
+      <c r="D217" s="60"/>
     </row>
     <row r="218" spans="1:4" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A218" s="77" t="s">
+      <c r="A218" s="76" t="s">
         <v>60</v>
       </c>
-      <c r="B218" s="78" t="s">
+      <c r="B218" s="77" t="s">
         <v>61</v>
       </c>
-      <c r="C218" s="79" t="s">
+      <c r="C218" s="78" t="s">
         <v>56</v>
       </c>
-      <c r="D218" s="65"/>
+      <c r="D218" s="64"/>
     </row>
     <row r="219" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A219" s="53"/>
-      <c r="B219" s="80"/>
-      <c r="C219" s="81"/>
-      <c r="D219" s="81"/>
+      <c r="A219" s="52"/>
+      <c r="B219" s="79"/>
+      <c r="C219" s="80"/>
+      <c r="D219" s="80"/>
     </row>
     <row r="220" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A220" s="54" t="s">
+      <c r="A220" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="B220" s="82"/>
-      <c r="C220" s="83"/>
-      <c r="D220" s="83"/>
+      <c r="B220" s="81"/>
+      <c r="C220" s="82"/>
+      <c r="D220" s="82"/>
     </row>
     <row r="221" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A221" s="55" t="s">
+      <c r="A221" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="B221" s="84" t="s">
+      <c r="B221" s="83" t="s">
         <v>64</v>
       </c>
-      <c r="C221" s="85" t="s">
+      <c r="C221" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="D221" s="57" t="s">
+      <c r="D221" s="56" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="222" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A222" s="67"/>
-      <c r="B222" s="68"/>
-      <c r="C222" s="99"/>
-      <c r="D222" s="100"/>
+      <c r="A222" s="66"/>
+      <c r="B222" s="67"/>
+      <c r="C222" s="98"/>
+      <c r="D222" s="99"/>
     </row>
     <row r="223" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A223" s="101"/>
-      <c r="B223" s="101"/>
-      <c r="C223" s="101"/>
-      <c r="D223" s="101"/>
+      <c r="A223" s="100"/>
+      <c r="B223" s="100"/>
+      <c r="C223" s="100"/>
+      <c r="D223" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A197:D197"/>
     <mergeCell ref="A141:D141"/>
-    <mergeCell ref="A169:D169"/>
-    <mergeCell ref="A197:D197"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A29:D29"/>
     <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A113:D113"/>
     <mergeCell ref="A85:D85"/>
-    <mergeCell ref="A113:D113"/>
+    <mergeCell ref="A169:D169"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
@@ -4572,7 +4711,7 @@
     </row>
     <row r="2" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Complete Sprint 3 portfolio evidence
</commit_message>
<xml_diff>
--- a/public/Integraal_Sprint_Logboek_Officieel.xlsx
+++ b/public/Integraal_Sprint_Logboek_Officieel.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasmijnmesu/Desktop/Mijn Projecten/Portfolio-Jasmijn-Mesu/public/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasmijnmesu/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E2A49F-CA74-6848-B436-A938A14A20AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{441C0961-207D-5247-B138-E2509004DABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17360" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3820" yWindow="760" windowWidth="25580" windowHeight="17360" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
     <sheet name="Logboek" sheetId="2" r:id="rId2"/>
     <sheet name="Lijsten" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="131">
   <si>
     <t>LU</t>
   </si>
@@ -415,6 +415,93 @@
   </si>
   <si>
     <t>O</t>
+  </si>
+  <si>
+    <t>1. Masterprompt: Een uitgebreide prompt met een vaste indeling van twaalf hoofdstukken, cover en samenvatting.
+2. Proefeditie: Een volledig magazine als HTML-mail over de periode 06-10 t/m 12-10-2026.
+3. Ontvangst: De mail is getest in Gmail op iPhone op leesbaarheid en volledigheid.
+4. Workflow: Een stappenplan met bronnen, taalmodel en verzending.</t>
+  </si>
+  <si>
+    <t>1. Promptstructuur: De prompt bevat een duidelijke rol, context, stappen, gewenst format en eisen.
+2. Verificatie: Links en feiten zijn gecontroleerd en gevonden fouten zijn vastgelegd.
+3. Transparantie: Duidelijk vermeld wat AI deed, wat eigen werk is en wat de grenzen zijn.
+4. E-mailkwaliteit: E-mailveilige HTML die onder de Gmail-limiet blijft.
+5. Herbruikbaarheid: Prompt en proces zijn over te zetten naar Make of n8n.</t>
+  </si>
+  <si>
+    <t>1. Website: Versie 3 is live en bereikbaar via een link.
+2. Webshop: Winkelwagen, prijzen, bestelknoppen en verkoopteksten zijn verwijderd.
+3. Portfolio: Het kopje "Over mij" is verwijderd en zijn werk staat centraal.
+4. Afbeeldingen: Uitsneden en verhoudingen zijn aangepast, zodat zijn ontwerpen goed zichtbaar zijn.
+5. Mobiel: Het menu werkt, teksten zijn leesbaar en er is geen horizontaal scrollen.
+6. Review: De website en het gebruik ervan zijn samen met Ronald doorgenomen en zijn feedback is vastgelegd.</t>
+  </si>
+  <si>
+    <t>1. Stijlconsistentie: Typografie en marges sluiten op elkaar aan en lettertype en logo van Ronald zijn behouden.
+2. Afbeeldingskwaliteit: Afbeeldingen zijn scherp, niet vervormd en geschikt voor het web.
+3. Bruikbaarheid: Zijn werk is vanaf de homepage in maximaal 1 klik bereikbaar.
+4. Leesbaarheid: Contrast en tekstgrootte zijn op mobiel goed.</t>
+  </si>
+  <si>
+    <t>1. Vergelijking: Een tabel met minimaal 5 cursussen van minimaal 3 aanbieders.
+2. Begrippen: Uitleg van het verschil tussen deelnamebewijs, badge, certificaat en officiële certificering.
+3. Selectie: Een onderbouwde top 3 van cursussen die ik ga volgen.
+4. Verslag en presentatie: Een kort onderzoeksverslag, gepresenteerd tijdens de Show &amp; Grow.</t>
+  </si>
+  <si>
+    <t>1. Criteria: Een vooraf vastgestelde matrix (relevantie, erkenning, kosten, tijd, niveau, bewijs van afronding).
+2. Triangulatie: AI-onderzoek is gecontroleerd op de officiële cursuspagina's.
+3. Transparantie: Gebruikte LLM's en prompts zijn vastgelegd in een bijlage.
+4. Bronvermelding: Bronnen zijn gecontroleerd en genoteerd volgens APA 7.</t>
+  </si>
+  <si>
+    <t>Suzanne Koppenhol</t>
+  </si>
+  <si>
+    <t>Ik heb mijn AI-agent (The Career Brief) getest en besproken met Suzanne Koppenhol. Zij heeft meerdere ervaringen met agents. Haar advies: om de agent echt goed te laten werken, is het verstandig om hem uit te breiden in Make of n8n, eventueel met een API-koppeling.</t>
+  </si>
+  <si>
+    <t>Ik neem dit advies mee naar sprint 4 en ga verder met Make of n8n en API-koppelingen.</t>
+  </si>
+  <si>
+    <t>Met The Career Brief heb ik onderzocht welke AI-ontwikkelingen invloed hebben op mijn toekomstige werk, bijvoorbeeld binnen projectmanagement, consultancy en business. Ik heb onderzocht welke onderwerpen relevant zijn en hoe AI het werk binnen organisaties verandert. Daarnaast heb ik onderzoek gedaan naar gratis AI-cursussen en certificaten om te bepalen welke vaardigheden ik zelf verder wil ontwikkelen. Hieruit concludeer ik dat AI-agents en automatisering voor mij belangrijke vaardigheden worden, omdat een agent al een groot deel van het onderzoekswerk kan overnemen. Daarom kies ik cursussen die hierop aansluiten.</t>
+  </si>
+  <si>
+    <t>Ik heb The Career Brief ontwikkeld: een AI-gestuurd weekmagazine dat nieuws onderzoekt en verwerkt in twaalf hoofdstukken. Ik heb de inhoud, schrijfstijl en vormgeving uitgewerkt en verschillende versies getest. De automatische verzending via Gmail werkt nog niet volledig. Daarnaast heb ik de website van Ronald Boiten verbeterd. Samen met hem heb ik de website doorgenomen, de winkelwagen verwijderd en de vormgeving meer op zijn werk afgestemd. Beide oplossingen presenteer ik tijdens het Show &amp; Grow-moment van deze sprint.</t>
+  </si>
+  <si>
+    <t>Bij The Career Brief heb ik aandacht besteed aan betrouwbare bronnen, het controleren van informatie en het verantwoord gebruiken van afbeeldingen. Ik heb hiervoor instructies opgenomen in mijn prompt. Het daadwerkelijk testen en beoordelen hiervan wil ik in een volgende sprint verder oppakken.</t>
+  </si>
+  <si>
+    <t>Voor de website van Ronald heb ik gewerkt met Claude Code en Visual Studio Code. Bij The Career Brief heb ik ChatGPT gebruikt om een uitgebreide masterprompt te ontwikkelen, taken in te plannen en nieuwsbrieven met HTML-opmaak via Gmail te testen. Daarbij ontdekte ik dat automatische verzending aanvullende koppelingen vraagt. Daarom ben ik mij ook gaan verdiepen in Make, n8n en API's.</t>
+  </si>
+  <si>
+    <t>Vanuit mijn eigen interesse om wekelijks op de hoogte te blijven van ontwikkelingen heb ik The Career Brief bedacht. Ik heb zelfstandig onderzocht hoe ik dit kon realiseren en de nieuwsbrief meerdere keren aangepast op basis van mijn testresultaten. Ook heb ik feedback gevraagd aan Suzanne Koppenhol, die ervaring heeft met AI-agents. Haar advies om met Make of n8n en API-koppelingen verder te werken neem ik mee naar sprint 4.</t>
+  </si>
+  <si>
+    <t>Als toekomstig project- en organisatieprofessional,
+wil ik een AI-workflow ontwikkelen die wekelijks zelfstandig actuele ontwikkelingen onderzoekt, betrouwbare bronnen selecteert en deze verwerkt tot een persoonlijk weekmagazine (The Career Brief), met twaalf vaste hoofdstukken, uitgebreide artikelen en een professionele opmaak,
+zodat ik op de hoogte blijf van ontwikkelingen binnen AI, business en mijn toekomstige werkveld en leer hoe ik AI-agents en automatisering kan inzetten om informatie te verzamelen, te verwerken en automatisch via Gmail te versturen.</t>
+  </si>
+  <si>
+    <t>Als webbouwer,
+wil ik de bestaande website van Ronald Boiten verder ontwikkelen tot een overzichtelijke en professionele portfoliowebsite, waarbij zijn ontwerpen centraal staan en zijn persoonlijke stijl beter terugkomt,
+zodat bezoekers een goed beeld krijgen van zijn werk en de website aansluit bij hoe Ronald zichzelf en zijn projecten wil presenteren.</t>
+  </si>
+  <si>
+    <t>Als student van de minor Futureproof met AI,
+wil ik onderzoeken welke gratis AI-cursussen en certificaten van erkende aanbieders aansluiten bij mijn interesses en toekomstige loopbaan,
+zodat ik een bewuste keuze kan maken over welke kennis en vaardigheden ik verder wil ontwikkelen en hoe ik hiermee mijn cv en LinkedIn-profiel kan versterken.</t>
+  </si>
+  <si>
+    <t>Deze sprint heb ik geleerd dat het ontwikkelen van een AI-toepassing verder gaat dan alleen een goede prompt schrijven. Bij The Career Brief ontdekte ik dat er aanvullende koppelingen nodig zijn om een nieuwsbrief volledig automatisch te versturen. Ook heb ik geleerd hoe ik AI kan gebruiken om een website te verbeteren op basis van feedback van een opdrachtgever. Door mijn onderzoek naar AI-cursussen heb ik daarnaast meer inzicht gekregen in welke vaardigheden ik zelf wil ontwikkelen.</t>
+  </si>
+  <si>
+    <t>Ik wil blijven werken aan projecten die aansluiten bij mijn eigen interesses en waarbij ik iets kan ontwikkelen dat daadwerkelijk gebruikt kan worden. Ook wil ik blijven testen, feedback vragen en mijn werk steeds verder verbeteren.</t>
+  </si>
+  <si>
+    <t>In de volgende sprint wil ik mij meer verdiepen in Make, n8n en API-koppelingen, zodat ik The Career Brief verder kan automatiseren. Daarnaast wil ik eerder controleren of mijn ideeën technisch haalbaar zijn en mijn onderzoek naar AI ook daadwerkelijk toepassen in de praktijk.</t>
   </si>
 </sst>
 </file>
@@ -423,7 +510,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="166" formatCode="dd\-mm\-yy"/>
+    <numFmt numFmtId="165" formatCode="dd\-mm\-yy"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -1306,13 +1393,13 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="7" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2090,7 +2177,7 @@
       </c>
       <c r="C2" s="8">
         <f>COUNTIF(D2:K2, "V")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="9" t="str">
         <f>Logboek!C18</f>
@@ -2102,7 +2189,7 @@
       </c>
       <c r="F2" s="9" t="str">
         <f>Logboek!C74</f>
-        <v>-</v>
+        <v>V</v>
       </c>
       <c r="G2" s="9" t="str">
         <f>Logboek!C102</f>
@@ -2134,7 +2221,7 @@
       </c>
       <c r="C3" s="8">
         <f>COUNTIF(D3:K3, "V")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3" s="9" t="str">
         <f>Logboek!C19</f>
@@ -2146,7 +2233,7 @@
       </c>
       <c r="F3" s="9" t="str">
         <f>Logboek!C75</f>
-        <v>-</v>
+        <v>V</v>
       </c>
       <c r="G3" s="9" t="str">
         <f>Logboek!C103</f>
@@ -2222,7 +2309,7 @@
       </c>
       <c r="C5" s="8">
         <f>COUNTIF(D5:K5, "V")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="9" t="str">
         <f>Logboek!C21</f>
@@ -2234,7 +2321,7 @@
       </c>
       <c r="F5" s="9" t="str">
         <f>Logboek!C77</f>
-        <v>-</v>
+        <v>V</v>
       </c>
       <c r="G5" s="9" t="str">
         <f>Logboek!C105</f>
@@ -2266,7 +2353,7 @@
       </c>
       <c r="C6" s="8">
         <f>COUNTIF(D6:K6, "V")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" s="9" t="str">
         <f>Logboek!C22</f>
@@ -2278,7 +2365,7 @@
       </c>
       <c r="F6" s="9" t="str">
         <f>Logboek!C78</f>
-        <v>-</v>
+        <v>V</v>
       </c>
       <c r="G6" s="9" t="str">
         <f>Logboek!C106</f>
@@ -2311,7 +2398,7 @@
       </c>
       <c r="C7" s="12">
         <f>SUM(D6:K7)</f>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D7" s="13">
         <f t="shared" ref="D7:K7" si="0">COUNTIF(D2:D6, "V")</f>
@@ -2323,7 +2410,7 @@
       </c>
       <c r="F7" s="13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G7" s="13">
         <f t="shared" si="0"/>
@@ -3036,42 +3123,46 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" ht="183" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A61" s="22" t="s">
         <v>30</v>
       </c>
       <c r="B61" s="25" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="C61" s="23" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D61" s="24" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="22"/>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="155" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="22" t="s">
+        <v>30</v>
+      </c>
       <c r="B62" s="25" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="C62" s="23" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D62" s="24" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="22"/>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="127" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="22" t="s">
+        <v>26</v>
+      </c>
       <c r="B63" s="25" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="C63" s="23" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="D63" s="24" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
@@ -3126,11 +3217,19 @@
         <v>42</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="31"/>
-      <c r="B69" s="23"/>
-      <c r="C69" s="23"/>
-      <c r="D69" s="24"/>
+    <row r="69" spans="1:4" ht="71" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="31">
+        <v>46303</v>
+      </c>
+      <c r="B69" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="C69" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="D69" s="24" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="70" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A70" s="35"/>
@@ -3166,7 +3265,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="74" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:4" ht="169" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A74" s="39" t="s">
         <v>47</v>
       </c>
@@ -3174,11 +3273,13 @@
         <v>48</v>
       </c>
       <c r="C74" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="D74" s="24"/>
-    </row>
-    <row r="75" spans="1:4" ht="28.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+      <c r="D74" s="24" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="141" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A75" s="39" t="s">
         <v>51</v>
       </c>
@@ -3186,11 +3287,13 @@
         <v>52</v>
       </c>
       <c r="C75" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="D75" s="24"/>
-    </row>
-    <row r="76" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+      <c r="D75" s="24" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="85" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A76" s="39" t="s">
         <v>54</v>
       </c>
@@ -3200,9 +3303,11 @@
       <c r="C76" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="D76" s="24"/>
-    </row>
-    <row r="77" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="D76" s="24" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="99" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A77" s="39" t="s">
         <v>57</v>
       </c>
@@ -3210,11 +3315,13 @@
         <v>58</v>
       </c>
       <c r="C77" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="D77" s="24"/>
-    </row>
-    <row r="78" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+      <c r="D77" s="24" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="113" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A78" s="41" t="s">
         <v>60</v>
       </c>
@@ -3222,9 +3329,11 @@
         <v>61</v>
       </c>
       <c r="C78" s="43" t="s">
-        <v>56</v>
-      </c>
-      <c r="D78" s="29"/>
+        <v>49</v>
+      </c>
+      <c r="D78" s="29" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="79" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A79" s="16"/>
@@ -3254,11 +3363,17 @@
         <v>66</v>
       </c>
     </row>
-    <row r="82" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4" ht="103" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A82" s="31"/>
-      <c r="B82" s="23"/>
-      <c r="C82" s="50"/>
-      <c r="D82" s="50"/>
+      <c r="B82" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="C82" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="D82" s="50" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="83" spans="1:4" ht="15" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A83" s="51"/>

</xml_diff>